<commit_message>
feat: add mini junction box item to PO-2609-001
</commit_message>
<xml_diff>
--- a/backups/warsgate_accounting_backup_2026-09-24.xlsx
+++ b/backups/warsgate_accounting_backup_2026-09-24.xlsx
@@ -704,7 +704,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -778,13 +778,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>prod-1</v>
+        <v>prod-box-minijb01</v>
       </c>
       <c r="B3" t="str">
-        <v>PLC-S7-1200</v>
+        <v>BOX-MINI-JB01</v>
       </c>
       <c r="C3" t="str">
-        <v>Siemens PLC SIMATIC S7-1200 CPU 1214C DC/DC/DC</v>
+        <v>mini junction box</v>
       </c>
       <c r="D3" t="str">
         <v>PRODUCT</v>
@@ -793,33 +793,33 @@
         <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F3" t="str">
-        <v>เครื่อง</v>
+        <v>Set</v>
       </c>
       <c r="G3">
-        <v>18500</v>
+        <v>300</v>
       </c>
       <c r="H3">
-        <v>13200</v>
+        <v>300</v>
       </c>
       <c r="I3">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K3" t="str">
-        <v>โปรแกรมเมเบิลคอนโทรลเลอร์ 14 DI / 10 DO / 2 AI</v>
+        <v>mini junction box</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>prod-2</v>
+        <v>prod-1</v>
       </c>
       <c r="B4" t="str">
-        <v>SERVO-750W</v>
+        <v>PLC-S7-1200</v>
       </c>
       <c r="C4" t="str">
-        <v>Omron Servo Motor &amp; Driver Set 750W 3000RPM</v>
+        <v>Siemens PLC SIMATIC S7-1200 CPU 1214C DC/DC/DC</v>
       </c>
       <c r="D4" t="str">
         <v>PRODUCT</v>
@@ -828,33 +828,33 @@
         <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F4" t="str">
-        <v>ชุด</v>
+        <v>เครื่อง</v>
       </c>
       <c r="G4">
-        <v>24500</v>
+        <v>18500</v>
       </c>
       <c r="H4">
-        <v>17800</v>
+        <v>13200</v>
       </c>
       <c r="I4">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K4" t="str">
-        <v>ชุดเซอร์โวมอเตอร์และไดรเวอร์ความแม่นยำสูง</v>
+        <v>โปรแกรมเมเบิลคอนโทรลเลอร์ 14 DI / 10 DO / 2 AI</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>prod-3</v>
+        <v>prod-2</v>
       </c>
       <c r="B5" t="str">
-        <v>HMI-KTP700</v>
+        <v>SERVO-750W</v>
       </c>
       <c r="C5" t="str">
-        <v>Siemens Touch Panel HMI KTP700 Basic 7 นิ้ว</v>
+        <v>Omron Servo Motor &amp; Driver Set 750W 3000RPM</v>
       </c>
       <c r="D5" t="str">
         <v>PRODUCT</v>
@@ -863,68 +863,68 @@
         <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F5" t="str">
-        <v>เครื่อง</v>
+        <v>ชุด</v>
       </c>
       <c r="G5">
-        <v>16800</v>
+        <v>24500</v>
       </c>
       <c r="H5">
-        <v>12100</v>
+        <v>17800</v>
       </c>
       <c r="I5">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K5" t="str">
-        <v>หน้าจอสัมผัสควบคุมเครื่องจักรความละเอียดสูง</v>
+        <v>ชุดเซอร์โวมอเตอร์และไดรเวอร์ความแม่นยำสูง</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>prod-4</v>
+        <v>prod-3</v>
       </c>
       <c r="B6" t="str">
-        <v>ENG-PROGRAMMING</v>
+        <v>HMI-KTP700</v>
       </c>
       <c r="C6" t="str">
-        <v>ค่าบริการเขียนโปรแกรม PLC / SCADA &amp; HMI Design</v>
+        <v>Siemens Touch Panel HMI KTP700 Basic 7 นิ้ว</v>
       </c>
       <c r="D6" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E6" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F6" t="str">
-        <v>Man-Day</v>
+        <v>เครื่อง</v>
       </c>
       <c r="G6">
-        <v>15000</v>
+        <v>16800</v>
       </c>
       <c r="H6">
-        <v>7500</v>
+        <v>12100</v>
       </c>
       <c r="I6">
-        <v>999</v>
+        <v>12</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K6" t="str">
-        <v>วิศวกรผู้เชี่ยวชาญออกแบบและพัฒนาโปรแกรมควบคุมไลน์ผลิต</v>
+        <v>หน้าจอสัมผัสควบคุมเครื่องจักรความละเอียดสูง</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>prod-5</v>
+        <v>prod-4</v>
       </c>
       <c r="B7" t="str">
-        <v>ENG-COMMISSION</v>
+        <v>ENG-PROGRAMMING</v>
       </c>
       <c r="C7" t="str">
-        <v>ค่าบริการทดสอบและติดตั้งระบบหน้างาน (On-site Commissioning)</v>
+        <v>ค่าบริการเขียนโปรแกรม PLC / SCADA &amp; HMI Design</v>
       </c>
       <c r="D7" t="str">
         <v>SERVICE</v>
@@ -936,10 +936,10 @@
         <v>Man-Day</v>
       </c>
       <c r="G7">
-        <v>12000</v>
+        <v>15000</v>
       </c>
       <c r="H7">
-        <v>6000</v>
+        <v>7500</v>
       </c>
       <c r="I7">
         <v>999</v>
@@ -948,33 +948,33 @@
         <v>0</v>
       </c>
       <c r="K7" t="str">
-        <v>ทดสอบความปลอดภัยและการทำงานของไลน์การผลิตหน้าโรงงาน</v>
+        <v>วิศวกรผู้เชี่ยวชาญออกแบบและพัฒนาโปรแกรมควบคุมไลน์ผลิต</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>prod-trace-1</v>
+        <v>prod-5</v>
       </c>
       <c r="B8" t="str">
-        <v>SW-TRACE-001</v>
+        <v>ENG-COMMISSION</v>
       </c>
       <c r="C8" t="str">
-        <v>Traceability Solenoid Line Software</v>
+        <v>ค่าบริการทดสอบและติดตั้งระบบหน้างาน (On-site Commissioning)</v>
       </c>
       <c r="D8" t="str">
         <v>SERVICE</v>
       </c>
       <c r="E8" t="str">
-        <v>SOFTWARE</v>
+        <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F8" t="str">
-        <v>Job</v>
+        <v>Man-Day</v>
       </c>
       <c r="G8">
-        <v>2023419</v>
+        <v>12000</v>
       </c>
       <c r="H8">
-        <v>850000</v>
+        <v>6000</v>
       </c>
       <c r="I8">
         <v>999</v>
@@ -983,18 +983,18 @@
         <v>0</v>
       </c>
       <c r="K8" t="str">
-        <v>ซอฟต์แวร์ระบบตรวจสอบย้อนกลับ (Traceability) สายการผลิต Solenoid Line</v>
+        <v>ทดสอบความปลอดภัยและการทำงานของไลน์การผลิตหน้าโรงงาน</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>prod-trace-2</v>
+        <v>prod-trace-1</v>
       </c>
       <c r="B9" t="str">
-        <v>SW-TRACE-002</v>
+        <v>SW-TRACE-001</v>
       </c>
       <c r="C9" t="str">
-        <v>Traceability Solenoid Line Software เพิ่มเติม</v>
+        <v>Traceability Solenoid Line Software</v>
       </c>
       <c r="D9" t="str">
         <v>SERVICE</v>
@@ -1006,10 +1006,10 @@
         <v>Job</v>
       </c>
       <c r="G9">
-        <v>150000</v>
+        <v>2023419</v>
       </c>
       <c r="H9">
-        <v>60000</v>
+        <v>850000</v>
       </c>
       <c r="I9">
         <v>999</v>
@@ -1018,33 +1018,33 @@
         <v>0</v>
       </c>
       <c r="K9" t="str">
-        <v>ซอฟต์แวร์ฟังก์ชันเพิ่มเติม Traceability Solenoid Line</v>
+        <v>ซอฟต์แวร์ระบบตรวจสอบย้อนกลับ (Traceability) สายการผลิต Solenoid Line</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>prod-6</v>
+        <v>prod-trace-2</v>
       </c>
       <c r="B10" t="str">
-        <v>MAINT-ANNUAL</v>
+        <v>SW-TRACE-002</v>
       </c>
       <c r="C10" t="str">
-        <v>สัญญาบริการบำรุงรักษาระบบอัตโนมัติรายปี (Annual PM Contract)</v>
+        <v>Traceability Solenoid Line Software เพิ่มเติม</v>
       </c>
       <c r="D10" t="str">
         <v>SERVICE</v>
       </c>
       <c r="E10" t="str">
-        <v>MAINTENANCE</v>
+        <v>SOFTWARE</v>
       </c>
       <c r="F10" t="str">
-        <v>สัญญา</v>
+        <v>Job</v>
       </c>
       <c r="G10">
-        <v>120000</v>
+        <v>150000</v>
       </c>
       <c r="H10">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="I10">
         <v>999</v>
@@ -1053,53 +1053,53 @@
         <v>0</v>
       </c>
       <c r="K10" t="str">
-        <v>เข้าตรวจเช็คระบบรายไตรมาส (4 ครั้ง/ปี) พร้อม On-call 24 ชม.</v>
+        <v>ซอฟต์แวร์ฟังก์ชันเพิ่มเติม Traceability Solenoid Line</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>prod-tsf-1</v>
+        <v>prod-6</v>
       </c>
       <c r="B11" t="str">
-        <v>TSF-ST-001</v>
+        <v>MAINT-ANNUAL</v>
       </c>
       <c r="C11" t="str">
-        <v>Station Stacker Foam</v>
+        <v>สัญญาบริการบำรุงรักษาระบบอัตโนมัติรายปี (Annual PM Contract)</v>
       </c>
       <c r="D11" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E11" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>MAINTENANCE</v>
       </c>
       <c r="F11" t="str">
-        <v>SET</v>
+        <v>สัญญา</v>
       </c>
       <c r="G11">
-        <v>765394</v>
+        <v>120000</v>
       </c>
       <c r="H11">
-        <v>420000</v>
+        <v>40000</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11" t="str">
-        <v>ชุดสถานีเรียงโฟมอัตโนมัติ (Station Stacker Foam) เครื่อง TSF1 Auto pack LM1</v>
+        <v>เข้าตรวจเช็คระบบรายไตรมาส (4 ครั้ง/ปี) พร้อม On-call 24 ชม.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>prod-tsf-2</v>
+        <v>prod-tsf-1</v>
       </c>
       <c r="B12" t="str">
-        <v>TSF-ST-002</v>
+        <v>TSF-ST-001</v>
       </c>
       <c r="C12" t="str">
-        <v>Station Open Bag &amp; Insert Foam</v>
+        <v>Station Stacker Foam</v>
       </c>
       <c r="D12" t="str">
         <v>PRODUCT</v>
@@ -1111,10 +1111,10 @@
         <v>SET</v>
       </c>
       <c r="G12">
-        <v>650215</v>
+        <v>765394</v>
       </c>
       <c r="H12">
-        <v>350000</v>
+        <v>420000</v>
       </c>
       <c r="I12">
         <v>1</v>
@@ -1123,18 +1123,18 @@
         <v>0</v>
       </c>
       <c r="K12" t="str">
-        <v>ชุดสถานีเปิดถุงและบรรจุโฟม (Station Open Bag &amp; Insert Foam)</v>
+        <v>ชุดสถานีเรียงโฟมอัตโนมัติ (Station Stacker Foam) เครื่อง TSF1 Auto pack LM1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>prod-tsf-3</v>
+        <v>prod-tsf-2</v>
       </c>
       <c r="B13" t="str">
-        <v>TSF-ST-003</v>
+        <v>TSF-ST-002</v>
       </c>
       <c r="C13" t="str">
-        <v>Station Pallet Stacker Foam</v>
+        <v>Station Open Bag &amp; Insert Foam</v>
       </c>
       <c r="D13" t="str">
         <v>PRODUCT</v>
@@ -1146,10 +1146,10 @@
         <v>SET</v>
       </c>
       <c r="G13">
-        <v>690391</v>
+        <v>650215</v>
       </c>
       <c r="H13">
-        <v>380000</v>
+        <v>350000</v>
       </c>
       <c r="I13">
         <v>1</v>
@@ -1158,18 +1158,18 @@
         <v>0</v>
       </c>
       <c r="K13" t="str">
-        <v>ชุดสถานีเรียงพาเลทโฟม (Station Pallet Stacker Foam)</v>
+        <v>ชุดสถานีเปิดถุงและบรรจุโฟม (Station Open Bag &amp; Insert Foam)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>prod-tsf-4</v>
+        <v>prod-tsf-3</v>
       </c>
       <c r="B14" t="str">
-        <v>TSF-ST-004</v>
+        <v>TSF-ST-003</v>
       </c>
       <c r="C14" t="str">
-        <v>Contron Box System</v>
+        <v>Station Pallet Stacker Foam</v>
       </c>
       <c r="D14" t="str">
         <v>PRODUCT</v>
@@ -1181,10 +1181,10 @@
         <v>SET</v>
       </c>
       <c r="G14">
-        <v>312000</v>
+        <v>690391</v>
       </c>
       <c r="H14">
-        <v>170000</v>
+        <v>380000</v>
       </c>
       <c r="I14">
         <v>1</v>
@@ -1193,33 +1193,33 @@
         <v>0</v>
       </c>
       <c r="K14" t="str">
-        <v>ตู้ควบคุมระบบไฟฟ้าและ PLC คอนโทรลเลอร์ (Control Box System)</v>
+        <v>ชุดสถานีเรียงพาเลทโฟม (Station Pallet Stacker Foam)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>prod-tsf-5</v>
+        <v>prod-tsf-4</v>
       </c>
       <c r="B15" t="str">
-        <v>TSF-SRV-001</v>
+        <v>TSF-ST-004</v>
       </c>
       <c r="C15" t="str">
-        <v>Manpower and labor cost</v>
+        <v>Contron Box System</v>
       </c>
       <c r="D15" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E15" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F15" t="str">
-        <v>JOB</v>
+        <v>SET</v>
       </c>
       <c r="G15">
-        <v>575000</v>
+        <v>312000</v>
       </c>
       <c r="H15">
-        <v>280000</v>
+        <v>170000</v>
       </c>
       <c r="I15">
         <v>1</v>
@@ -1228,18 +1228,18 @@
         <v>0</v>
       </c>
       <c r="K15" t="str">
-        <v>ค่าแรงวิศวกร ประกอบ ติดตั้ง และทดสอบระบบ TSF1 Auto pack LM1</v>
+        <v>ตู้ควบคุมระบบไฟฟ้าและ PLC คอนโทรลเลอร์ (Control Box System)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>prod-tsf-6</v>
+        <v>prod-tsf-5</v>
       </c>
       <c r="B16" t="str">
-        <v>TSF-SRV-002</v>
+        <v>TSF-SRV-001</v>
       </c>
       <c r="C16" t="str">
-        <v>Transportation and accommodation</v>
+        <v>Manpower and labor cost</v>
       </c>
       <c r="D16" t="str">
         <v>SERVICE</v>
@@ -1251,10 +1251,10 @@
         <v>JOB</v>
       </c>
       <c r="G16">
-        <v>45000</v>
+        <v>575000</v>
       </c>
       <c r="H16">
-        <v>30000</v>
+        <v>280000</v>
       </c>
       <c r="I16">
         <v>1</v>
@@ -1263,18 +1263,18 @@
         <v>0</v>
       </c>
       <c r="K16" t="str">
-        <v>ค่าขนส่งเครื่องจักรและค่าที่พักเดินทางหน้างานโรงงานชลบุรี</v>
+        <v>ค่าแรงวิศวกร ประกอบ ติดตั้ง และทดสอบระบบ TSF1 Auto pack LM1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>prod-tsf-7</v>
+        <v>prod-tsf-6</v>
       </c>
       <c r="B17" t="str">
-        <v>TSF-SRV-003</v>
+        <v>TSF-SRV-002</v>
       </c>
       <c r="C17" t="str">
-        <v>Profit / Project Management &amp; Warranty 1 year</v>
+        <v>Transportation and accommodation</v>
       </c>
       <c r="D17" t="str">
         <v>SERVICE</v>
@@ -1286,10 +1286,10 @@
         <v>JOB</v>
       </c>
       <c r="G17">
-        <v>607600</v>
+        <v>45000</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="I17">
         <v>1</v>
@@ -1298,53 +1298,53 @@
         <v>0</v>
       </c>
       <c r="K17" t="str">
-        <v>ค่าบริหารโครงการ บริการหลังการขาย และรับประกันระบบ 1 ปี (Warranty 1 year)</v>
+        <v>ค่าขนส่งเครื่องจักรและค่าที่พักเดินทางหน้างานโรงงานชลบุรี</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>prod-pnp-corr</v>
+        <v>prod-tsf-7</v>
       </c>
       <c r="B18" t="str">
-        <v>SW-TRACE-CORR</v>
+        <v>TSF-SRV-003</v>
       </c>
       <c r="C18" t="str">
-        <v>Traceability Corrugating Line</v>
+        <v>Profit / Project Management &amp; Warranty 1 year</v>
       </c>
       <c r="D18" t="str">
         <v>SERVICE</v>
       </c>
       <c r="E18" t="str">
-        <v>SOFTWARE</v>
+        <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F18" t="str">
-        <v>Job</v>
+        <v>JOB</v>
       </c>
       <c r="G18">
-        <v>1005002.64</v>
+        <v>607600</v>
       </c>
       <c r="H18">
-        <v>450000</v>
+        <v>0</v>
       </c>
       <c r="I18">
-        <v>999</v>
+        <v>1</v>
       </c>
       <c r="J18">
         <v>0</v>
       </c>
       <c r="K18" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Corrugating Line โครงการ Fujipart (PO: 2505004)</v>
+        <v>ค่าบริหารโครงการ บริการหลังการขาย และรับประกันระบบ 1 ปี (Warranty 1 year)</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>prod-pnp-wind</v>
+        <v>prod-pnp-corr</v>
       </c>
       <c r="B19" t="str">
-        <v>SW-TRACE-WIND</v>
+        <v>SW-TRACE-CORR</v>
       </c>
       <c r="C19" t="str">
-        <v>Traceability Winding Line</v>
+        <v>Traceability Corrugating Line</v>
       </c>
       <c r="D19" t="str">
         <v>SERVICE</v>
@@ -1356,10 +1356,10 @@
         <v>Job</v>
       </c>
       <c r="G19">
-        <v>707304.38</v>
+        <v>1005002.64</v>
       </c>
       <c r="H19">
-        <v>320000</v>
+        <v>450000</v>
       </c>
       <c r="I19">
         <v>999</v>
@@ -1368,18 +1368,18 @@
         <v>0</v>
       </c>
       <c r="K19" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Winding Line โครงการ Fujipart (PO: 2505004)</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Corrugating Line โครงการ Fujipart (PO: 2505004)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>prod-pnp-adh</v>
+        <v>prod-pnp-wind</v>
       </c>
       <c r="B20" t="str">
-        <v>SW-TRACE-ADH</v>
+        <v>SW-TRACE-WIND</v>
       </c>
       <c r="C20" t="str">
-        <v>Traceability Adhesive &amp; Spin Winding Line</v>
+        <v>Traceability Winding Line</v>
       </c>
       <c r="D20" t="str">
         <v>SERVICE</v>
@@ -1391,10 +1391,10 @@
         <v>Job</v>
       </c>
       <c r="G20">
-        <v>874426.94</v>
+        <v>707304.38</v>
       </c>
       <c r="H20">
-        <v>390000</v>
+        <v>320000</v>
       </c>
       <c r="I20">
         <v>999</v>
@@ -1403,18 +1403,18 @@
         <v>0</v>
       </c>
       <c r="K20" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Adhesive &amp; Spin Winding Line โครงการ Fujipart (PO: 2505004)</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Winding Line โครงการ Fujipart (PO: 2505004)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>prod-pnp-df4</v>
+        <v>prod-pnp-adh</v>
       </c>
       <c r="B21" t="str">
-        <v>SW-TRACE-DF4</v>
+        <v>SW-TRACE-ADH</v>
       </c>
       <c r="C21" t="str">
-        <v>Traceability DF4 Line</v>
+        <v>Traceability Adhesive &amp; Spin Winding Line</v>
       </c>
       <c r="D21" t="str">
         <v>SERVICE</v>
@@ -1426,10 +1426,10 @@
         <v>Job</v>
       </c>
       <c r="G21">
-        <v>1203060.14</v>
+        <v>874426.94</v>
       </c>
       <c r="H21">
-        <v>540000</v>
+        <v>390000</v>
       </c>
       <c r="I21">
         <v>999</v>
@@ -1438,18 +1438,18 @@
         <v>0</v>
       </c>
       <c r="K21" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต DF4 Line โครงการ Fujipart (PO: 2505004)</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Adhesive &amp; Spin Winding Line โครงการ Fujipart (PO: 2505004)</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>prod-pnp-pack</v>
+        <v>prod-pnp-df4</v>
       </c>
       <c r="B22" t="str">
-        <v>SW-TRACE-PACK</v>
+        <v>SW-TRACE-DF4</v>
       </c>
       <c r="C22" t="str">
-        <v>Traceability Packing Line</v>
+        <v>Traceability DF4 Line</v>
       </c>
       <c r="D22" t="str">
         <v>SERVICE</v>
@@ -1461,10 +1461,10 @@
         <v>Job</v>
       </c>
       <c r="G22">
-        <v>553196.28</v>
+        <v>1203060.14</v>
       </c>
       <c r="H22">
-        <v>250000</v>
+        <v>540000</v>
       </c>
       <c r="I22">
         <v>999</v>
@@ -1473,68 +1473,68 @@
         <v>0</v>
       </c>
       <c r="K22" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Packing Line โครงการ Fujipart (PO: 2505004)</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต DF4 Line โครงการ Fujipart (PO: 2505004)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>prod-pnp-fab</v>
+        <v>prod-pnp-pack</v>
       </c>
       <c r="B23" t="str">
-        <v>PNP-FAB-001</v>
+        <v>SW-TRACE-PACK</v>
       </c>
       <c r="C23" t="str">
-        <v>Standard and Feb Part (Zone 1-6)</v>
+        <v>Traceability Packing Line</v>
       </c>
       <c r="D23" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E23" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>SOFTWARE</v>
       </c>
       <c r="F23" t="str">
-        <v>Set</v>
+        <v>Job</v>
       </c>
       <c r="G23">
-        <v>1140000</v>
+        <v>553196.28</v>
       </c>
       <c r="H23">
-        <v>650000</v>
+        <v>250000</v>
       </c>
       <c r="I23">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="J23">
         <v>0</v>
       </c>
       <c r="K23" t="str">
-        <v>ชุดโครงสร้างมาตรฐานและชิ้นงานประกอบ Fabricated Parts Zone 1-6 (PO: 2605001)</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Packing Line โครงการ Fujipart (PO: 2505004)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>prod-pnp-labor-z</v>
+        <v>prod-pnp-fab</v>
       </c>
       <c r="B24" t="str">
-        <v>PNP-LAB-001</v>
+        <v>PNP-FAB-001</v>
       </c>
       <c r="C24" t="str">
-        <v>Manpower and Labor Cost (Zone 1-6)</v>
+        <v>Standard and Feb Part (Zone 1-6)</v>
       </c>
       <c r="D24" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E24" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F24" t="str">
-        <v>Job</v>
+        <v>Set</v>
       </c>
       <c r="G24">
-        <v>670000</v>
+        <v>1140000</v>
       </c>
       <c r="H24">
-        <v>350000</v>
+        <v>650000</v>
       </c>
       <c r="I24">
         <v>1</v>
@@ -1543,18 +1543,18 @@
         <v>0</v>
       </c>
       <c r="K24" t="str">
-        <v>ค่าแรงวิศวกรและทีมช่างประกอบ ติดตั้ง ทดสอบ Zone 1-6 (PO: 2605001)</v>
+        <v>ชุดโครงสร้างมาตรฐานและชิ้นงานประกอบ Fabricated Parts Zone 1-6 (PO: 2605001)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>prod-pnp-trans-z</v>
+        <v>prod-pnp-labor-z</v>
       </c>
       <c r="B25" t="str">
-        <v>PNP-LOG-001</v>
+        <v>PNP-LAB-001</v>
       </c>
       <c r="C25" t="str">
-        <v>Transportation and accommodation (Zone 1-6)</v>
+        <v>Manpower and Labor Cost (Zone 1-6)</v>
       </c>
       <c r="D25" t="str">
         <v>SERVICE</v>
@@ -1563,13 +1563,13 @@
         <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F25" t="str">
-        <v>EA</v>
+        <v>Job</v>
       </c>
       <c r="G25">
-        <v>45000</v>
+        <v>670000</v>
       </c>
       <c r="H25">
-        <v>30000</v>
+        <v>350000</v>
       </c>
       <c r="I25">
         <v>1</v>
@@ -1578,18 +1578,18 @@
         <v>0</v>
       </c>
       <c r="K25" t="str">
-        <v>ค่าขนส่งและที่พักเดินทางหน้างาน Zone 1-6 (PO: 2605001)</v>
+        <v>ค่าแรงวิศวกรและทีมช่างประกอบ ติดตั้ง ทดสอบ Zone 1-6 (PO: 2605001)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>prod-pnp-pm-z</v>
+        <v>prod-pnp-trans-z</v>
       </c>
       <c r="B26" t="str">
-        <v>PNP-PM-001</v>
+        <v>PNP-LOG-001</v>
       </c>
       <c r="C26" t="str">
-        <v>Project Management (Zone 1-6)</v>
+        <v>Transportation and accommodation (Zone 1-6)</v>
       </c>
       <c r="D26" t="str">
         <v>SERVICE</v>
@@ -1601,10 +1601,10 @@
         <v>EA</v>
       </c>
       <c r="G26">
-        <v>556500</v>
+        <v>45000</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="I26">
         <v>1</v>
@@ -1613,33 +1613,33 @@
         <v>0</v>
       </c>
       <c r="K26" t="str">
-        <v>ค่าบริหารจัดการโครงการ ควบคุมงาน และทดสอบระบบ Zone 1-6 (PO: 2605001)</v>
+        <v>ค่าขนส่งและที่พักเดินทางหน้างาน Zone 1-6 (PO: 2605001)</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>prod-pnp-fab-z7</v>
+        <v>prod-pnp-pm-z</v>
       </c>
       <c r="B27" t="str">
-        <v>PNP-FAB-002</v>
+        <v>PNP-PM-001</v>
       </c>
       <c r="C27" t="str">
-        <v>Standard and Feb Part (Zone 7)</v>
+        <v>Project Management (Zone 1-6)</v>
       </c>
       <c r="D27" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E27" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F27" t="str">
-        <v>Set</v>
+        <v>EA</v>
       </c>
       <c r="G27">
-        <v>641000</v>
+        <v>556500</v>
       </c>
       <c r="H27">
-        <v>350000</v>
+        <v>0</v>
       </c>
       <c r="I27">
         <v>1</v>
@@ -1648,33 +1648,33 @@
         <v>0</v>
       </c>
       <c r="K27" t="str">
-        <v>ชุดโครงสร้างมาตรฐานและชิ้นงานประกอบ Fabricated Parts Zone 7 (PO: 2605002)</v>
+        <v>ค่าบริหารจัดการโครงการ ควบคุมงาน และทดสอบระบบ Zone 1-6 (PO: 2605001)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>prod-pnp-labor-z7</v>
+        <v>prod-pnp-fab-z7</v>
       </c>
       <c r="B28" t="str">
-        <v>PNP-LAB-002</v>
+        <v>PNP-FAB-002</v>
       </c>
       <c r="C28" t="str">
-        <v>Manpower and Labor Cost (Zone 7)</v>
+        <v>Standard and Feb Part (Zone 7)</v>
       </c>
       <c r="D28" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E28" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F28" t="str">
-        <v>Job</v>
+        <v>Set</v>
       </c>
       <c r="G28">
-        <v>220000</v>
+        <v>641000</v>
       </c>
       <c r="H28">
-        <v>110000</v>
+        <v>350000</v>
       </c>
       <c r="I28">
         <v>1</v>
@@ -1683,18 +1683,18 @@
         <v>0</v>
       </c>
       <c r="K28" t="str">
-        <v>ค่าแรงวิศวกรและทีมช่างประกอบ ติดตั้ง ทดสอบ Zone 7 (PO: 2605002)</v>
+        <v>ชุดโครงสร้างมาตรฐานและชิ้นงานประกอบ Fabricated Parts Zone 7 (PO: 2605002)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>prod-pnp-trans-z7</v>
+        <v>prod-pnp-labor-z7</v>
       </c>
       <c r="B29" t="str">
-        <v>PNP-LOG-002</v>
+        <v>PNP-LAB-002</v>
       </c>
       <c r="C29" t="str">
-        <v>Transportation and accommodation (Zone 7)</v>
+        <v>Manpower and Labor Cost (Zone 7)</v>
       </c>
       <c r="D29" t="str">
         <v>SERVICE</v>
@@ -1703,13 +1703,13 @@
         <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F29" t="str">
-        <v>EA</v>
+        <v>Job</v>
       </c>
       <c r="G29">
-        <v>45000</v>
+        <v>220000</v>
       </c>
       <c r="H29">
-        <v>30000</v>
+        <v>110000</v>
       </c>
       <c r="I29">
         <v>1</v>
@@ -1718,18 +1718,18 @@
         <v>0</v>
       </c>
       <c r="K29" t="str">
-        <v>ค่าขนส่งและที่พักเดินทางหน้างาน Zone 7 (PO: 2605002)</v>
+        <v>ค่าแรงวิศวกรและทีมช่างประกอบ ติดตั้ง ทดสอบ Zone 7 (PO: 2605002)</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>prod-pnp-pm-z7</v>
+        <v>prod-pnp-trans-z7</v>
       </c>
       <c r="B30" t="str">
-        <v>PNP-PM-002</v>
+        <v>PNP-LOG-002</v>
       </c>
       <c r="C30" t="str">
-        <v>Project Management (Zone 7)</v>
+        <v>Transportation and accommodation (Zone 7)</v>
       </c>
       <c r="D30" t="str">
         <v>SERVICE</v>
@@ -1741,10 +1741,10 @@
         <v>EA</v>
       </c>
       <c r="G30">
-        <v>271800</v>
+        <v>45000</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="I30">
         <v>1</v>
@@ -1753,53 +1753,53 @@
         <v>0</v>
       </c>
       <c r="K30" t="str">
-        <v>ค่าบริหารจัดการโครงการ ควบคุมงาน และทดสอบระบบ Zone 7 (PO: 2605002)</v>
+        <v>ค่าขนส่งและที่พักเดินทางหน้างาน Zone 7 (PO: 2605002)</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>prod-pnp-plc-eth</v>
+        <v>prod-pnp-pm-z7</v>
       </c>
       <c r="B31" t="str">
-        <v>PLC-ETH-001</v>
+        <v>PNP-PM-002</v>
       </c>
       <c r="C31" t="str">
-        <v>PLC Control Board (Ethernet IP)</v>
+        <v>Project Management (Zone 7)</v>
       </c>
       <c r="D31" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E31" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F31" t="str">
         <v>EA</v>
       </c>
       <c r="G31">
-        <v>35040</v>
+        <v>271800</v>
       </c>
       <c r="H31">
-        <v>22000</v>
+        <v>0</v>
       </c>
       <c r="I31">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="J31">
         <v>0</v>
       </c>
       <c r="K31" t="str">
-        <v>บอร์ดควบคุม PLC รองรับการเชื่อมต่อเครือข่าย Ethernet IP (PO: 2607001)</v>
+        <v>ค่าบริหารจัดการโครงการ ควบคุมงาน และทดสอบระบบ Zone 7 (PO: 2605002)</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>prod-pnp-sub-plc</v>
+        <v>prod-pnp-plc-eth</v>
       </c>
       <c r="B32" t="str">
-        <v>PLC-SUB-001</v>
+        <v>PLC-ETH-001</v>
       </c>
       <c r="C32" t="str">
-        <v>Sub PLC Box + Aceessories</v>
+        <v>PLC Control Board (Ethernet IP)</v>
       </c>
       <c r="D32" t="str">
         <v>PRODUCT</v>
@@ -1811,30 +1811,30 @@
         <v>EA</v>
       </c>
       <c r="G32">
-        <v>26000</v>
+        <v>35040</v>
       </c>
       <c r="H32">
-        <v>15000</v>
+        <v>22000</v>
       </c>
       <c r="I32">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="J32">
         <v>0</v>
       </c>
       <c r="K32" t="str">
-        <v>ตู้ Sub PLC พร้อมอุปกรณ์ส่วนควบ Accessories (PO: 2607001)</v>
+        <v>บอร์ดควบคุม PLC รองรับการเชื่อมต่อเครือข่าย Ethernet IP (PO: 2607001)</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>prod-pnp-rack-pc</v>
+        <v>prod-pnp-sub-plc</v>
       </c>
       <c r="B33" t="str">
-        <v>PC-RACK-001</v>
+        <v>PLC-SUB-001</v>
       </c>
       <c r="C33" t="str">
-        <v>Rack PC Center</v>
+        <v>Sub PLC Box + Aceessories</v>
       </c>
       <c r="D33" t="str">
         <v>PRODUCT</v>
@@ -1846,45 +1846,45 @@
         <v>EA</v>
       </c>
       <c r="G33">
-        <v>12000</v>
+        <v>26000</v>
       </c>
       <c r="H33">
-        <v>7000</v>
+        <v>15000</v>
       </c>
       <c r="I33">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J33">
         <v>0</v>
       </c>
       <c r="K33" t="str">
-        <v>ตู้แร็คศูนย์คอมพิวเตอร์และเซิร์ฟเวอร์ Rack PC Center (PO: 2607001)</v>
+        <v>ตู้ Sub PLC พร้อมอุปกรณ์ส่วนควบ Accessories (PO: 2607001)</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>prod-pnp-plc-dc</v>
+        <v>prod-pnp-rack-pc</v>
       </c>
       <c r="B34" t="str">
-        <v>PLC-DC-001</v>
+        <v>PC-RACK-001</v>
       </c>
       <c r="C34" t="str">
-        <v>PLC Data Center Line</v>
+        <v>Rack PC Center</v>
       </c>
       <c r="D34" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E34" t="str">
-        <v>SOFTWARE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F34" t="str">
         <v>EA</v>
       </c>
       <c r="G34">
-        <v>150000</v>
+        <v>12000</v>
       </c>
       <c r="H34">
-        <v>80000</v>
+        <v>7000</v>
       </c>
       <c r="I34">
         <v>1</v>
@@ -1893,33 +1893,33 @@
         <v>0</v>
       </c>
       <c r="K34" t="str">
-        <v>ระบบศูนย์รวมและประมวลผลข้อมูลสายการผลิต PLC Data Center Line (PO: 2607001)</v>
+        <v>ตู้แร็คศูนย์คอมพิวเตอร์และเซิร์ฟเวอร์ Rack PC Center (PO: 2607001)</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>prod-pnp-struct-sup</v>
+        <v>prod-pnp-plc-dc</v>
       </c>
       <c r="B35" t="str">
-        <v>STR-SUP-001</v>
+        <v>PLC-DC-001</v>
       </c>
       <c r="C35" t="str">
-        <v>Stucture Support</v>
+        <v>PLC Data Center Line</v>
       </c>
       <c r="D35" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E35" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>SOFTWARE</v>
       </c>
       <c r="F35" t="str">
         <v>EA</v>
       </c>
       <c r="G35">
-        <v>20000</v>
+        <v>150000</v>
       </c>
       <c r="H35">
-        <v>10000</v>
+        <v>80000</v>
       </c>
       <c r="I35">
         <v>1</v>
@@ -1928,18 +1928,18 @@
         <v>0</v>
       </c>
       <c r="K35" t="str">
-        <v>ชุดโครงสร้างรองรับและฐานยึดอุปกรณ์ Structure Support (PO: 2607001)</v>
+        <v>ระบบศูนย์รวมและประมวลผลข้อมูลสายการผลิต PLC Data Center Line (PO: 2607001)</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>prod-pnp-pc-center</v>
+        <v>prod-pnp-struct-sup</v>
       </c>
       <c r="B36" t="str">
-        <v>PC-CTR-001</v>
+        <v>STR-SUP-001</v>
       </c>
       <c r="C36" t="str">
-        <v>PC Center</v>
+        <v>Stucture Support</v>
       </c>
       <c r="D36" t="str">
         <v>PRODUCT</v>
@@ -1951,10 +1951,10 @@
         <v>EA</v>
       </c>
       <c r="G36">
-        <v>123000</v>
+        <v>20000</v>
       </c>
       <c r="H36">
-        <v>75000</v>
+        <v>10000</v>
       </c>
       <c r="I36">
         <v>1</v>
@@ -1963,47 +1963,82 @@
         <v>0</v>
       </c>
       <c r="K36" t="str">
-        <v>เครื่องคอมพิวเตอร์แม่ข่ายประมวลผล PC Center (PO: 2607001)</v>
+        <v>ชุดโครงสร้างรองรับและฐานยึดอุปกรณ์ Structure Support (PO: 2607001)</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>prod-pnp-pm-2607</v>
+        <v>prod-pnp-pc-center</v>
       </c>
       <c r="B37" t="str">
-        <v>PNP-PM-2607</v>
+        <v>PC-CTR-001</v>
       </c>
       <c r="C37" t="str">
-        <v>Project Management (PO: 2607001)</v>
+        <v>PC Center</v>
       </c>
       <c r="D37" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E37" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F37" t="str">
         <v>EA</v>
       </c>
       <c r="G37">
+        <v>123000</v>
+      </c>
+      <c r="H37">
+        <v>75000</v>
+      </c>
+      <c r="I37">
+        <v>1</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37" t="str">
+        <v>เครื่องคอมพิวเตอร์แม่ข่ายประมวลผล PC Center (PO: 2607001)</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>prod-pnp-pm-2607</v>
+      </c>
+      <c r="B38" t="str">
+        <v>PNP-PM-2607</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Project Management (PO: 2607001)</v>
+      </c>
+      <c r="D38" t="str">
+        <v>SERVICE</v>
+      </c>
+      <c r="E38" t="str">
+        <v>ENGINEERING_SERVICE</v>
+      </c>
+      <c r="F38" t="str">
+        <v>EA</v>
+      </c>
+      <c r="G38">
         <v>573552</v>
       </c>
-      <c r="H37">
-        <v>0</v>
-      </c>
-      <c r="I37">
-        <v>1</v>
-      </c>
-      <c r="J37">
-        <v>0</v>
-      </c>
-      <c r="K37" t="str">
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>1</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38" t="str">
         <v>ค่าบริหารจัดการโครงการ ควบคุมงาน และทดสอบระบบ (PO: 2607001)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3104,19 +3139,19 @@
         <v>2026-10-24</v>
       </c>
       <c r="I27">
-        <v>16500</v>
+        <v>21000</v>
       </c>
       <c r="J27">
-        <v>1155</v>
+        <v>1470</v>
       </c>
       <c r="K27">
-        <v>17655</v>
+        <v>22470</v>
       </c>
       <c r="L27">
         <v>0</v>
       </c>
       <c r="M27">
-        <v>17655</v>
+        <v>22470</v>
       </c>
       <c r="N27" t="str">
         <v>APPROVED</v>
@@ -3137,7 +3172,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L94"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5794,9 +5829,38 @@
         <v>0</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>PO-2609-001</v>
+      </c>
+      <c r="B94" t="str">
+        <v>PURCHASE_ORDER</v>
+      </c>
+      <c r="C94" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="E94">
+        <v>2</v>
+      </c>
+      <c r="F94" t="str">
+        <v/>
+      </c>
+      <c r="G94" t="str">
+        <v>mini junction box</v>
+      </c>
+      <c r="H94">
+        <v>15</v>
+      </c>
+      <c r="I94" t="str">
+        <v>Set</v>
+      </c>
+      <c r="K94">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L93"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L94"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: update pricePerUnit of item 1 to 300 in PO-2609-001
</commit_message>
<xml_diff>
--- a/backups/warsgate_accounting_backup_2026-09-24.xlsx
+++ b/backups/warsgate_accounting_backup_2026-09-24.xlsx
@@ -761,10 +761,10 @@
         <v>Set</v>
       </c>
       <c r="G2">
-        <v>1100</v>
+        <v>300</v>
       </c>
       <c r="H2">
-        <v>1100</v>
+        <v>300</v>
       </c>
       <c r="I2">
         <v>15</v>
@@ -3139,19 +3139,19 @@
         <v>2026-10-24</v>
       </c>
       <c r="I27">
-        <v>21000</v>
+        <v>9000</v>
       </c>
       <c r="J27">
-        <v>1470</v>
+        <v>630</v>
       </c>
       <c r="K27">
-        <v>22470</v>
+        <v>9630</v>
       </c>
       <c r="L27">
         <v>0</v>
       </c>
       <c r="M27">
-        <v>22470</v>
+        <v>9630</v>
       </c>
       <c r="N27" t="str">
         <v>APPROVED</v>

</xml_diff>

<commit_message>
feat: add quotation QT-2609-001 for PNP Technology Great OR Board project
</commit_message>
<xml_diff>
--- a/backups/warsgate_accounting_backup_2026-09-24.xlsx
+++ b/backups/warsgate_accounting_backup_2026-09-24.xlsx
@@ -503,7 +503,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -621,83 +621,45 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>cont-4</v>
+        <v>cont-ptech-1</v>
       </c>
       <c r="B4" t="str">
         <v>ซัพพลายเออร์ (Supplier)</v>
       </c>
       <c r="C4" t="str">
-        <v>คุณอารียา สุขสันต์</v>
+        <v>ฝ่ายขาย / ประสานงานขาย</v>
       </c>
       <c r="D4" t="str">
-        <v>บริษัท ออมรอน อีเลคทรอนิกส์ (ประเทศไทย) จำกัด</v>
+        <v>บริษัท พี-เทค แอนด์ คอนซัลติ้ง จำกัด</v>
       </c>
       <c r="E4" t="str">
-        <v>0105533088991</v>
+        <v>0105568020018</v>
       </c>
       <c r="F4" t="str">
         <v>00000</v>
       </c>
       <c r="G4" t="str">
-        <v>55 อาคารอาคเนย์ประกันภัย ชั้น 10 ถนนสีลม แขวงสุริยวงศ์ เขตบางรัก กรุงเทพฯ 10500</v>
+        <v>234/107 ถนน01 กาญจนาภิเษก แขวงสามวาตะวันตก เขตคลองสามวา กรุงเทพมหานคร 10510</v>
       </c>
       <c r="H4" t="str">
-        <v>02-637-5100</v>
+        <v>+(66) 81 184 6590</v>
       </c>
       <c r="I4" t="str">
-        <v>omron_thailand@omron.com</v>
+        <v>saintentex@gmail.com</v>
       </c>
       <c r="J4">
         <v>30</v>
       </c>
       <c r="K4">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="L4">
-        <v>94000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>cont-ptech-1</v>
-      </c>
-      <c r="B5" t="str">
-        <v>ซัพพลายเออร์ (Supplier)</v>
-      </c>
-      <c r="C5" t="str">
-        <v>ฝ่ายขาย / ประสานงานขาย</v>
-      </c>
-      <c r="D5" t="str">
-        <v>บริษัท พี-เทค แอนด์ คอนซัลติ้ง จำกัด</v>
-      </c>
-      <c r="E5" t="str">
-        <v>0105568020018</v>
-      </c>
-      <c r="F5" t="str">
-        <v>00000</v>
-      </c>
-      <c r="G5" t="str">
-        <v>234/107 ถนน01 กาญจนาภิเษก แขวงสามวาตะวันตก เขตคลองสามวา กรุงเทพมหานคร 10510</v>
-      </c>
-      <c r="H5" t="str">
-        <v>+(66) 81 184 6590</v>
-      </c>
-      <c r="I5" t="str">
-        <v>saintentex@gmail.com</v>
-      </c>
-      <c r="J5">
-        <v>30</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -743,13 +705,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>prod-spindle-01</v>
+        <v>prod-1</v>
       </c>
       <c r="B2" t="str">
-        <v>SPINDLE-ROLL-01</v>
+        <v>PLC-S7-1200</v>
       </c>
       <c r="C2" t="str">
-        <v>Roller Paper Printer Spindle (แกนหมุนกระดาษเครื่องพิมพ์อัปเกรด)</v>
+        <v>Siemens PLC SIMATIC S7-1200 CPU 1214C DC/DC/DC</v>
       </c>
       <c r="D2" t="str">
         <v>PRODUCT</v>
@@ -758,33 +720,33 @@
         <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F2" t="str">
-        <v>Set</v>
+        <v>เครื่อง</v>
       </c>
       <c r="G2">
-        <v>300</v>
+        <v>18500</v>
       </c>
       <c r="H2">
-        <v>300</v>
+        <v>13200</v>
       </c>
       <c r="I2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K2" t="str">
-        <v>แกนหมุนกระดาษเครื่องพิมพ์อัปเกรด (Roller Paper Printer Spindle)</v>
+        <v>โปรแกรมเมเบิลคอนโทรลเลอร์ 14 DI / 10 DO / 2 AI</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>prod-box-minijb01</v>
+        <v>prod-2</v>
       </c>
       <c r="B3" t="str">
-        <v>BOX-MINI-JB01</v>
+        <v>SERVO-750W</v>
       </c>
       <c r="C3" t="str">
-        <v>mini junction box</v>
+        <v>Omron Servo Motor &amp; Driver Set 750W 3000RPM</v>
       </c>
       <c r="D3" t="str">
         <v>PRODUCT</v>
@@ -793,33 +755,33 @@
         <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F3" t="str">
-        <v>Set</v>
+        <v>ชุด</v>
       </c>
       <c r="G3">
-        <v>300</v>
+        <v>24500</v>
       </c>
       <c r="H3">
-        <v>300</v>
+        <v>17800</v>
       </c>
       <c r="I3">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K3" t="str">
-        <v>mini junction box</v>
+        <v>ชุดเซอร์โวมอเตอร์และไดรเวอร์ความแม่นยำสูง</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>prod-1</v>
+        <v>prod-3</v>
       </c>
       <c r="B4" t="str">
-        <v>PLC-S7-1200</v>
+        <v>HMI-KTP700</v>
       </c>
       <c r="C4" t="str">
-        <v>Siemens PLC SIMATIC S7-1200 CPU 1214C DC/DC/DC</v>
+        <v>Siemens Touch Panel HMI KTP700 Basic 7 นิ้ว</v>
       </c>
       <c r="D4" t="str">
         <v>PRODUCT</v>
@@ -831,115 +793,115 @@
         <v>เครื่อง</v>
       </c>
       <c r="G4">
-        <v>18500</v>
+        <v>16800</v>
       </c>
       <c r="H4">
-        <v>13200</v>
+        <v>12100</v>
       </c>
       <c r="I4">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K4" t="str">
-        <v>โปรแกรมเมเบิลคอนโทรลเลอร์ 14 DI / 10 DO / 2 AI</v>
+        <v>หน้าจอสัมผัสควบคุมเครื่องจักรความละเอียดสูง</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>prod-2</v>
+        <v>prod-4</v>
       </c>
       <c r="B5" t="str">
-        <v>SERVO-750W</v>
+        <v>ENG-PROGRAMMING</v>
       </c>
       <c r="C5" t="str">
-        <v>Omron Servo Motor &amp; Driver Set 750W 3000RPM</v>
+        <v>ค่าบริการเขียนโปรแกรม PLC / SCADA &amp; HMI Design</v>
       </c>
       <c r="D5" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E5" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F5" t="str">
-        <v>ชุด</v>
+        <v>Man-Day</v>
       </c>
       <c r="G5">
-        <v>24500</v>
+        <v>15000</v>
       </c>
       <c r="H5">
-        <v>17800</v>
+        <v>7500</v>
       </c>
       <c r="I5">
-        <v>8</v>
+        <v>999</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K5" t="str">
-        <v>ชุดเซอร์โวมอเตอร์และไดรเวอร์ความแม่นยำสูง</v>
+        <v>วิศวกรผู้เชี่ยวชาญออกแบบและพัฒนาโปรแกรมควบคุมไลน์ผลิต</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>prod-3</v>
+        <v>prod-5</v>
       </c>
       <c r="B6" t="str">
-        <v>HMI-KTP700</v>
+        <v>ENG-COMMISSION</v>
       </c>
       <c r="C6" t="str">
-        <v>Siemens Touch Panel HMI KTP700 Basic 7 นิ้ว</v>
+        <v>ค่าบริการทดสอบและติดตั้งระบบหน้างาน (On-site Commissioning)</v>
       </c>
       <c r="D6" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E6" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F6" t="str">
-        <v>เครื่อง</v>
+        <v>Man-Day</v>
       </c>
       <c r="G6">
-        <v>16800</v>
+        <v>12000</v>
       </c>
       <c r="H6">
-        <v>12100</v>
+        <v>6000</v>
       </c>
       <c r="I6">
-        <v>12</v>
+        <v>999</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K6" t="str">
-        <v>หน้าจอสัมผัสควบคุมเครื่องจักรความละเอียดสูง</v>
+        <v>ทดสอบความปลอดภัยและการทำงานของไลน์การผลิตหน้าโรงงาน</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>prod-4</v>
+        <v>prod-trace-1</v>
       </c>
       <c r="B7" t="str">
-        <v>ENG-PROGRAMMING</v>
+        <v>SW-TRACE-001</v>
       </c>
       <c r="C7" t="str">
-        <v>ค่าบริการเขียนโปรแกรม PLC / SCADA &amp; HMI Design</v>
+        <v>Traceability Solenoid Line Software</v>
       </c>
       <c r="D7" t="str">
         <v>SERVICE</v>
       </c>
       <c r="E7" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>SOFTWARE</v>
       </c>
       <c r="F7" t="str">
-        <v>Man-Day</v>
+        <v>Job</v>
       </c>
       <c r="G7">
-        <v>15000</v>
+        <v>2023419</v>
       </c>
       <c r="H7">
-        <v>7500</v>
+        <v>850000</v>
       </c>
       <c r="I7">
         <v>999</v>
@@ -948,33 +910,33 @@
         <v>0</v>
       </c>
       <c r="K7" t="str">
-        <v>วิศวกรผู้เชี่ยวชาญออกแบบและพัฒนาโปรแกรมควบคุมไลน์ผลิต</v>
+        <v>ซอฟต์แวร์ระบบตรวจสอบย้อนกลับ (Traceability) สายการผลิต Solenoid Line</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>prod-5</v>
+        <v>prod-trace-2</v>
       </c>
       <c r="B8" t="str">
-        <v>ENG-COMMISSION</v>
+        <v>SW-TRACE-002</v>
       </c>
       <c r="C8" t="str">
-        <v>ค่าบริการทดสอบและติดตั้งระบบหน้างาน (On-site Commissioning)</v>
+        <v>Traceability Solenoid Line Software เพิ่มเติม</v>
       </c>
       <c r="D8" t="str">
         <v>SERVICE</v>
       </c>
       <c r="E8" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>SOFTWARE</v>
       </c>
       <c r="F8" t="str">
-        <v>Man-Day</v>
+        <v>Job</v>
       </c>
       <c r="G8">
-        <v>12000</v>
+        <v>150000</v>
       </c>
       <c r="H8">
-        <v>6000</v>
+        <v>60000</v>
       </c>
       <c r="I8">
         <v>999</v>
@@ -983,33 +945,33 @@
         <v>0</v>
       </c>
       <c r="K8" t="str">
-        <v>ทดสอบความปลอดภัยและการทำงานของไลน์การผลิตหน้าโรงงาน</v>
+        <v>ซอฟต์แวร์ฟังก์ชันเพิ่มเติม Traceability Solenoid Line</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>prod-trace-1</v>
+        <v>prod-6</v>
       </c>
       <c r="B9" t="str">
-        <v>SW-TRACE-001</v>
+        <v>MAINT-ANNUAL</v>
       </c>
       <c r="C9" t="str">
-        <v>Traceability Solenoid Line Software</v>
+        <v>สัญญาบริการบำรุงรักษาระบบอัตโนมัติรายปี (Annual PM Contract)</v>
       </c>
       <c r="D9" t="str">
         <v>SERVICE</v>
       </c>
       <c r="E9" t="str">
-        <v>SOFTWARE</v>
+        <v>MAINTENANCE</v>
       </c>
       <c r="F9" t="str">
-        <v>Job</v>
+        <v>สัญญา</v>
       </c>
       <c r="G9">
-        <v>2023419</v>
+        <v>120000</v>
       </c>
       <c r="H9">
-        <v>850000</v>
+        <v>40000</v>
       </c>
       <c r="I9">
         <v>999</v>
@@ -1018,88 +980,88 @@
         <v>0</v>
       </c>
       <c r="K9" t="str">
-        <v>ซอฟต์แวร์ระบบตรวจสอบย้อนกลับ (Traceability) สายการผลิต Solenoid Line</v>
+        <v>เข้าตรวจเช็คระบบรายไตรมาส (4 ครั้ง/ปี) พร้อม On-call 24 ชม.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>prod-trace-2</v>
+        <v>prod-tsf-1</v>
       </c>
       <c r="B10" t="str">
-        <v>SW-TRACE-002</v>
+        <v>TSF-ST-001</v>
       </c>
       <c r="C10" t="str">
-        <v>Traceability Solenoid Line Software เพิ่มเติม</v>
+        <v>Station Stacker Foam</v>
       </c>
       <c r="D10" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E10" t="str">
-        <v>SOFTWARE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F10" t="str">
-        <v>Job</v>
+        <v>SET</v>
       </c>
       <c r="G10">
-        <v>150000</v>
+        <v>765394</v>
       </c>
       <c r="H10">
-        <v>60000</v>
+        <v>420000</v>
       </c>
       <c r="I10">
-        <v>999</v>
+        <v>1</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10" t="str">
-        <v>ซอฟต์แวร์ฟังก์ชันเพิ่มเติม Traceability Solenoid Line</v>
+        <v>ชุดสถานีเรียงโฟมอัตโนมัติ (Station Stacker Foam) เครื่อง TSF1 Auto pack LM1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>prod-6</v>
+        <v>prod-tsf-2</v>
       </c>
       <c r="B11" t="str">
-        <v>MAINT-ANNUAL</v>
+        <v>TSF-ST-002</v>
       </c>
       <c r="C11" t="str">
-        <v>สัญญาบริการบำรุงรักษาระบบอัตโนมัติรายปี (Annual PM Contract)</v>
+        <v>Station Open Bag &amp; Insert Foam</v>
       </c>
       <c r="D11" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E11" t="str">
-        <v>MAINTENANCE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F11" t="str">
-        <v>สัญญา</v>
+        <v>SET</v>
       </c>
       <c r="G11">
-        <v>120000</v>
+        <v>650215</v>
       </c>
       <c r="H11">
-        <v>40000</v>
+        <v>350000</v>
       </c>
       <c r="I11">
-        <v>999</v>
+        <v>1</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11" t="str">
-        <v>เข้าตรวจเช็คระบบรายไตรมาส (4 ครั้ง/ปี) พร้อม On-call 24 ชม.</v>
+        <v>ชุดสถานีเปิดถุงและบรรจุโฟม (Station Open Bag &amp; Insert Foam)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>prod-tsf-1</v>
+        <v>prod-tsf-3</v>
       </c>
       <c r="B12" t="str">
-        <v>TSF-ST-001</v>
+        <v>TSF-ST-003</v>
       </c>
       <c r="C12" t="str">
-        <v>Station Stacker Foam</v>
+        <v>Station Pallet Stacker Foam</v>
       </c>
       <c r="D12" t="str">
         <v>PRODUCT</v>
@@ -1111,10 +1073,10 @@
         <v>SET</v>
       </c>
       <c r="G12">
-        <v>765394</v>
+        <v>690391</v>
       </c>
       <c r="H12">
-        <v>420000</v>
+        <v>380000</v>
       </c>
       <c r="I12">
         <v>1</v>
@@ -1123,18 +1085,18 @@
         <v>0</v>
       </c>
       <c r="K12" t="str">
-        <v>ชุดสถานีเรียงโฟมอัตโนมัติ (Station Stacker Foam) เครื่อง TSF1 Auto pack LM1</v>
+        <v>ชุดสถานีเรียงพาเลทโฟม (Station Pallet Stacker Foam)</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>prod-tsf-2</v>
+        <v>prod-tsf-4</v>
       </c>
       <c r="B13" t="str">
-        <v>TSF-ST-002</v>
+        <v>TSF-ST-004</v>
       </c>
       <c r="C13" t="str">
-        <v>Station Open Bag &amp; Insert Foam</v>
+        <v>Contron Box System</v>
       </c>
       <c r="D13" t="str">
         <v>PRODUCT</v>
@@ -1146,10 +1108,10 @@
         <v>SET</v>
       </c>
       <c r="G13">
-        <v>650215</v>
+        <v>312000</v>
       </c>
       <c r="H13">
-        <v>350000</v>
+        <v>170000</v>
       </c>
       <c r="I13">
         <v>1</v>
@@ -1158,33 +1120,33 @@
         <v>0</v>
       </c>
       <c r="K13" t="str">
-        <v>ชุดสถานีเปิดถุงและบรรจุโฟม (Station Open Bag &amp; Insert Foam)</v>
+        <v>ตู้ควบคุมระบบไฟฟ้าและ PLC คอนโทรลเลอร์ (Control Box System)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>prod-tsf-3</v>
+        <v>prod-tsf-5</v>
       </c>
       <c r="B14" t="str">
-        <v>TSF-ST-003</v>
+        <v>TSF-SRV-001</v>
       </c>
       <c r="C14" t="str">
-        <v>Station Pallet Stacker Foam</v>
+        <v>Manpower and labor cost</v>
       </c>
       <c r="D14" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E14" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F14" t="str">
-        <v>SET</v>
+        <v>JOB</v>
       </c>
       <c r="G14">
-        <v>690391</v>
+        <v>575000</v>
       </c>
       <c r="H14">
-        <v>380000</v>
+        <v>280000</v>
       </c>
       <c r="I14">
         <v>1</v>
@@ -1193,33 +1155,33 @@
         <v>0</v>
       </c>
       <c r="K14" t="str">
-        <v>ชุดสถานีเรียงพาเลทโฟม (Station Pallet Stacker Foam)</v>
+        <v>ค่าแรงวิศวกร ประกอบ ติดตั้ง และทดสอบระบบ TSF1 Auto pack LM1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>prod-tsf-4</v>
+        <v>prod-tsf-6</v>
       </c>
       <c r="B15" t="str">
-        <v>TSF-ST-004</v>
+        <v>TSF-SRV-002</v>
       </c>
       <c r="C15" t="str">
-        <v>Contron Box System</v>
+        <v>Transportation and accommodation</v>
       </c>
       <c r="D15" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E15" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F15" t="str">
-        <v>SET</v>
+        <v>JOB</v>
       </c>
       <c r="G15">
-        <v>312000</v>
+        <v>45000</v>
       </c>
       <c r="H15">
-        <v>170000</v>
+        <v>30000</v>
       </c>
       <c r="I15">
         <v>1</v>
@@ -1228,18 +1190,18 @@
         <v>0</v>
       </c>
       <c r="K15" t="str">
-        <v>ตู้ควบคุมระบบไฟฟ้าและ PLC คอนโทรลเลอร์ (Control Box System)</v>
+        <v>ค่าขนส่งเครื่องจักรและค่าที่พักเดินทางหน้างานโรงงานชลบุรี</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>prod-tsf-5</v>
+        <v>prod-tsf-7</v>
       </c>
       <c r="B16" t="str">
-        <v>TSF-SRV-001</v>
+        <v>TSF-SRV-003</v>
       </c>
       <c r="C16" t="str">
-        <v>Manpower and labor cost</v>
+        <v>Profit / Project Management &amp; Warranty 1 year</v>
       </c>
       <c r="D16" t="str">
         <v>SERVICE</v>
@@ -1251,10 +1213,10 @@
         <v>JOB</v>
       </c>
       <c r="G16">
-        <v>575000</v>
+        <v>607600</v>
       </c>
       <c r="H16">
-        <v>280000</v>
+        <v>0</v>
       </c>
       <c r="I16">
         <v>1</v>
@@ -1263,88 +1225,88 @@
         <v>0</v>
       </c>
       <c r="K16" t="str">
-        <v>ค่าแรงวิศวกร ประกอบ ติดตั้ง และทดสอบระบบ TSF1 Auto pack LM1</v>
+        <v>ค่าบริหารโครงการ บริการหลังการขาย และรับประกันระบบ 1 ปี (Warranty 1 year)</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>prod-tsf-6</v>
+        <v>prod-pnp-corr</v>
       </c>
       <c r="B17" t="str">
-        <v>TSF-SRV-002</v>
+        <v>SW-TRACE-CORR</v>
       </c>
       <c r="C17" t="str">
-        <v>Transportation and accommodation</v>
+        <v>Traceability Corrugating Line</v>
       </c>
       <c r="D17" t="str">
         <v>SERVICE</v>
       </c>
       <c r="E17" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>SOFTWARE</v>
       </c>
       <c r="F17" t="str">
-        <v>JOB</v>
+        <v>Job</v>
       </c>
       <c r="G17">
-        <v>45000</v>
+        <v>1005002.64</v>
       </c>
       <c r="H17">
-        <v>30000</v>
+        <v>450000</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="J17">
         <v>0</v>
       </c>
       <c r="K17" t="str">
-        <v>ค่าขนส่งเครื่องจักรและค่าที่พักเดินทางหน้างานโรงงานชลบุรี</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Corrugating Line โครงการ Fujipart (PO: 2505004)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>prod-tsf-7</v>
+        <v>prod-pnp-wind</v>
       </c>
       <c r="B18" t="str">
-        <v>TSF-SRV-003</v>
+        <v>SW-TRACE-WIND</v>
       </c>
       <c r="C18" t="str">
-        <v>Profit / Project Management &amp; Warranty 1 year</v>
+        <v>Traceability Winding Line</v>
       </c>
       <c r="D18" t="str">
         <v>SERVICE</v>
       </c>
       <c r="E18" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>SOFTWARE</v>
       </c>
       <c r="F18" t="str">
-        <v>JOB</v>
+        <v>Job</v>
       </c>
       <c r="G18">
-        <v>607600</v>
+        <v>707304.38</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>320000</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>999</v>
       </c>
       <c r="J18">
         <v>0</v>
       </c>
       <c r="K18" t="str">
-        <v>ค่าบริหารโครงการ บริการหลังการขาย และรับประกันระบบ 1 ปี (Warranty 1 year)</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Winding Line โครงการ Fujipart (PO: 2505004)</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>prod-pnp-corr</v>
+        <v>prod-pnp-adh</v>
       </c>
       <c r="B19" t="str">
-        <v>SW-TRACE-CORR</v>
+        <v>SW-TRACE-ADH</v>
       </c>
       <c r="C19" t="str">
-        <v>Traceability Corrugating Line</v>
+        <v>Traceability Adhesive &amp; Spin Winding Line</v>
       </c>
       <c r="D19" t="str">
         <v>SERVICE</v>
@@ -1356,10 +1318,10 @@
         <v>Job</v>
       </c>
       <c r="G19">
-        <v>1005002.64</v>
+        <v>874426.94</v>
       </c>
       <c r="H19">
-        <v>450000</v>
+        <v>390000</v>
       </c>
       <c r="I19">
         <v>999</v>
@@ -1368,18 +1330,18 @@
         <v>0</v>
       </c>
       <c r="K19" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Corrugating Line โครงการ Fujipart (PO: 2505004)</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Adhesive &amp; Spin Winding Line โครงการ Fujipart (PO: 2505004)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>prod-pnp-wind</v>
+        <v>prod-pnp-df4</v>
       </c>
       <c r="B20" t="str">
-        <v>SW-TRACE-WIND</v>
+        <v>SW-TRACE-DF4</v>
       </c>
       <c r="C20" t="str">
-        <v>Traceability Winding Line</v>
+        <v>Traceability DF4 Line</v>
       </c>
       <c r="D20" t="str">
         <v>SERVICE</v>
@@ -1391,10 +1353,10 @@
         <v>Job</v>
       </c>
       <c r="G20">
-        <v>707304.38</v>
+        <v>1203060.14</v>
       </c>
       <c r="H20">
-        <v>320000</v>
+        <v>540000</v>
       </c>
       <c r="I20">
         <v>999</v>
@@ -1403,18 +1365,18 @@
         <v>0</v>
       </c>
       <c r="K20" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Winding Line โครงการ Fujipart (PO: 2505004)</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต DF4 Line โครงการ Fujipart (PO: 2505004)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>prod-pnp-adh</v>
+        <v>prod-pnp-pack</v>
       </c>
       <c r="B21" t="str">
-        <v>SW-TRACE-ADH</v>
+        <v>SW-TRACE-PACK</v>
       </c>
       <c r="C21" t="str">
-        <v>Traceability Adhesive &amp; Spin Winding Line</v>
+        <v>Traceability Packing Line</v>
       </c>
       <c r="D21" t="str">
         <v>SERVICE</v>
@@ -1426,10 +1388,10 @@
         <v>Job</v>
       </c>
       <c r="G21">
-        <v>874426.94</v>
+        <v>553196.28</v>
       </c>
       <c r="H21">
-        <v>390000</v>
+        <v>250000</v>
       </c>
       <c r="I21">
         <v>999</v>
@@ -1438,103 +1400,103 @@
         <v>0</v>
       </c>
       <c r="K21" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Adhesive &amp; Spin Winding Line โครงการ Fujipart (PO: 2505004)</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Packing Line โครงการ Fujipart (PO: 2505004)</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>prod-pnp-df4</v>
+        <v>prod-pnp-fab</v>
       </c>
       <c r="B22" t="str">
-        <v>SW-TRACE-DF4</v>
+        <v>PNP-FAB-001</v>
       </c>
       <c r="C22" t="str">
-        <v>Traceability DF4 Line</v>
+        <v>Standard and Feb Part (Zone 1-6)</v>
       </c>
       <c r="D22" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E22" t="str">
-        <v>SOFTWARE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F22" t="str">
-        <v>Job</v>
+        <v>Set</v>
       </c>
       <c r="G22">
-        <v>1203060.14</v>
+        <v>1140000</v>
       </c>
       <c r="H22">
-        <v>540000</v>
+        <v>650000</v>
       </c>
       <c r="I22">
-        <v>999</v>
+        <v>1</v>
       </c>
       <c r="J22">
         <v>0</v>
       </c>
       <c r="K22" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต DF4 Line โครงการ Fujipart (PO: 2505004)</v>
+        <v>ชุดโครงสร้างมาตรฐานและชิ้นงานประกอบ Fabricated Parts Zone 1-6 (PO: 2605001)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>prod-pnp-pack</v>
+        <v>prod-pnp-labor-z</v>
       </c>
       <c r="B23" t="str">
-        <v>SW-TRACE-PACK</v>
+        <v>PNP-LAB-001</v>
       </c>
       <c r="C23" t="str">
-        <v>Traceability Packing Line</v>
+        <v>Manpower and Labor Cost (Zone 1-6)</v>
       </c>
       <c r="D23" t="str">
         <v>SERVICE</v>
       </c>
       <c r="E23" t="str">
-        <v>SOFTWARE</v>
+        <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F23" t="str">
         <v>Job</v>
       </c>
       <c r="G23">
-        <v>553196.28</v>
+        <v>670000</v>
       </c>
       <c r="H23">
-        <v>250000</v>
+        <v>350000</v>
       </c>
       <c r="I23">
-        <v>999</v>
+        <v>1</v>
       </c>
       <c r="J23">
         <v>0</v>
       </c>
       <c r="K23" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Packing Line โครงการ Fujipart (PO: 2505004)</v>
+        <v>ค่าแรงวิศวกรและทีมช่างประกอบ ติดตั้ง ทดสอบ Zone 1-6 (PO: 2605001)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>prod-pnp-fab</v>
+        <v>prod-pnp-trans-z</v>
       </c>
       <c r="B24" t="str">
-        <v>PNP-FAB-001</v>
+        <v>PNP-LOG-001</v>
       </c>
       <c r="C24" t="str">
-        <v>Standard and Feb Part (Zone 1-6)</v>
+        <v>Transportation and accommodation (Zone 1-6)</v>
       </c>
       <c r="D24" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E24" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F24" t="str">
-        <v>Set</v>
+        <v>EA</v>
       </c>
       <c r="G24">
-        <v>1140000</v>
+        <v>45000</v>
       </c>
       <c r="H24">
-        <v>650000</v>
+        <v>30000</v>
       </c>
       <c r="I24">
         <v>1</v>
@@ -1543,18 +1505,18 @@
         <v>0</v>
       </c>
       <c r="K24" t="str">
-        <v>ชุดโครงสร้างมาตรฐานและชิ้นงานประกอบ Fabricated Parts Zone 1-6 (PO: 2605001)</v>
+        <v>ค่าขนส่งและที่พักเดินทางหน้างาน Zone 1-6 (PO: 2605001)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>prod-pnp-labor-z</v>
+        <v>prod-pnp-pm-z</v>
       </c>
       <c r="B25" t="str">
-        <v>PNP-LAB-001</v>
+        <v>PNP-PM-001</v>
       </c>
       <c r="C25" t="str">
-        <v>Manpower and Labor Cost (Zone 1-6)</v>
+        <v>Project Management (Zone 1-6)</v>
       </c>
       <c r="D25" t="str">
         <v>SERVICE</v>
@@ -1563,13 +1525,13 @@
         <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F25" t="str">
-        <v>Job</v>
+        <v>EA</v>
       </c>
       <c r="G25">
-        <v>670000</v>
+        <v>556500</v>
       </c>
       <c r="H25">
-        <v>350000</v>
+        <v>0</v>
       </c>
       <c r="I25">
         <v>1</v>
@@ -1578,33 +1540,33 @@
         <v>0</v>
       </c>
       <c r="K25" t="str">
-        <v>ค่าแรงวิศวกรและทีมช่างประกอบ ติดตั้ง ทดสอบ Zone 1-6 (PO: 2605001)</v>
+        <v>ค่าบริหารจัดการโครงการ ควบคุมงาน และทดสอบระบบ Zone 1-6 (PO: 2605001)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>prod-pnp-trans-z</v>
+        <v>prod-pnp-fab-z7</v>
       </c>
       <c r="B26" t="str">
-        <v>PNP-LOG-001</v>
+        <v>PNP-FAB-002</v>
       </c>
       <c r="C26" t="str">
-        <v>Transportation and accommodation (Zone 1-6)</v>
+        <v>Standard and Feb Part (Zone 7)</v>
       </c>
       <c r="D26" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E26" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F26" t="str">
-        <v>EA</v>
+        <v>Set</v>
       </c>
       <c r="G26">
-        <v>45000</v>
+        <v>641000</v>
       </c>
       <c r="H26">
-        <v>30000</v>
+        <v>350000</v>
       </c>
       <c r="I26">
         <v>1</v>
@@ -1613,18 +1575,18 @@
         <v>0</v>
       </c>
       <c r="K26" t="str">
-        <v>ค่าขนส่งและที่พักเดินทางหน้างาน Zone 1-6 (PO: 2605001)</v>
+        <v>ชุดโครงสร้างมาตรฐานและชิ้นงานประกอบ Fabricated Parts Zone 7 (PO: 2605002)</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>prod-pnp-pm-z</v>
+        <v>prod-pnp-labor-z7</v>
       </c>
       <c r="B27" t="str">
-        <v>PNP-PM-001</v>
+        <v>PNP-LAB-002</v>
       </c>
       <c r="C27" t="str">
-        <v>Project Management (Zone 1-6)</v>
+        <v>Manpower and Labor Cost (Zone 7)</v>
       </c>
       <c r="D27" t="str">
         <v>SERVICE</v>
@@ -1633,13 +1595,13 @@
         <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F27" t="str">
-        <v>EA</v>
+        <v>Job</v>
       </c>
       <c r="G27">
-        <v>556500</v>
+        <v>220000</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>110000</v>
       </c>
       <c r="I27">
         <v>1</v>
@@ -1648,33 +1610,33 @@
         <v>0</v>
       </c>
       <c r="K27" t="str">
-        <v>ค่าบริหารจัดการโครงการ ควบคุมงาน และทดสอบระบบ Zone 1-6 (PO: 2605001)</v>
+        <v>ค่าแรงวิศวกรและทีมช่างประกอบ ติดตั้ง ทดสอบ Zone 7 (PO: 2605002)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>prod-pnp-fab-z7</v>
+        <v>prod-pnp-trans-z7</v>
       </c>
       <c r="B28" t="str">
-        <v>PNP-FAB-002</v>
+        <v>PNP-LOG-002</v>
       </c>
       <c r="C28" t="str">
-        <v>Standard and Feb Part (Zone 7)</v>
+        <v>Transportation and accommodation (Zone 7)</v>
       </c>
       <c r="D28" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E28" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F28" t="str">
-        <v>Set</v>
+        <v>EA</v>
       </c>
       <c r="G28">
-        <v>641000</v>
+        <v>45000</v>
       </c>
       <c r="H28">
-        <v>350000</v>
+        <v>30000</v>
       </c>
       <c r="I28">
         <v>1</v>
@@ -1683,18 +1645,18 @@
         <v>0</v>
       </c>
       <c r="K28" t="str">
-        <v>ชุดโครงสร้างมาตรฐานและชิ้นงานประกอบ Fabricated Parts Zone 7 (PO: 2605002)</v>
+        <v>ค่าขนส่งและที่พักเดินทางหน้างาน Zone 7 (PO: 2605002)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>prod-pnp-labor-z7</v>
+        <v>prod-pnp-pm-z7</v>
       </c>
       <c r="B29" t="str">
-        <v>PNP-LAB-002</v>
+        <v>PNP-PM-002</v>
       </c>
       <c r="C29" t="str">
-        <v>Manpower and Labor Cost (Zone 7)</v>
+        <v>Project Management (Zone 7)</v>
       </c>
       <c r="D29" t="str">
         <v>SERVICE</v>
@@ -1703,13 +1665,13 @@
         <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F29" t="str">
-        <v>Job</v>
+        <v>EA</v>
       </c>
       <c r="G29">
-        <v>220000</v>
+        <v>271800</v>
       </c>
       <c r="H29">
-        <v>110000</v>
+        <v>0</v>
       </c>
       <c r="I29">
         <v>1</v>
@@ -1718,88 +1680,88 @@
         <v>0</v>
       </c>
       <c r="K29" t="str">
-        <v>ค่าแรงวิศวกรและทีมช่างประกอบ ติดตั้ง ทดสอบ Zone 7 (PO: 2605002)</v>
+        <v>ค่าบริหารจัดการโครงการ ควบคุมงาน และทดสอบระบบ Zone 7 (PO: 2605002)</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>prod-pnp-trans-z7</v>
+        <v>prod-pnp-plc-eth</v>
       </c>
       <c r="B30" t="str">
-        <v>PNP-LOG-002</v>
+        <v>PLC-ETH-001</v>
       </c>
       <c r="C30" t="str">
-        <v>Transportation and accommodation (Zone 7)</v>
+        <v>PLC Control Board (Ethernet IP)</v>
       </c>
       <c r="D30" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E30" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F30" t="str">
         <v>EA</v>
       </c>
       <c r="G30">
-        <v>45000</v>
+        <v>35040</v>
       </c>
       <c r="H30">
-        <v>30000</v>
+        <v>22000</v>
       </c>
       <c r="I30">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="J30">
         <v>0</v>
       </c>
       <c r="K30" t="str">
-        <v>ค่าขนส่งและที่พักเดินทางหน้างาน Zone 7 (PO: 2605002)</v>
+        <v>บอร์ดควบคุม PLC รองรับการเชื่อมต่อเครือข่าย Ethernet IP (PO: 2607001)</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>prod-pnp-pm-z7</v>
+        <v>prod-pnp-sub-plc</v>
       </c>
       <c r="B31" t="str">
-        <v>PNP-PM-002</v>
+        <v>PLC-SUB-001</v>
       </c>
       <c r="C31" t="str">
-        <v>Project Management (Zone 7)</v>
+        <v>Sub PLC Box + Aceessories</v>
       </c>
       <c r="D31" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E31" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F31" t="str">
         <v>EA</v>
       </c>
       <c r="G31">
-        <v>271800</v>
+        <v>26000</v>
       </c>
       <c r="H31">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="I31">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J31">
         <v>0</v>
       </c>
       <c r="K31" t="str">
-        <v>ค่าบริหารจัดการโครงการ ควบคุมงาน และทดสอบระบบ Zone 7 (PO: 2605002)</v>
+        <v>ตู้ Sub PLC พร้อมอุปกรณ์ส่วนควบ Accessories (PO: 2607001)</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>prod-pnp-plc-eth</v>
+        <v>prod-pnp-rack-pc</v>
       </c>
       <c r="B32" t="str">
-        <v>PLC-ETH-001</v>
+        <v>PC-RACK-001</v>
       </c>
       <c r="C32" t="str">
-        <v>PLC Control Board (Ethernet IP)</v>
+        <v>Rack PC Center</v>
       </c>
       <c r="D32" t="str">
         <v>PRODUCT</v>
@@ -1811,65 +1773,65 @@
         <v>EA</v>
       </c>
       <c r="G32">
-        <v>35040</v>
+        <v>12000</v>
       </c>
       <c r="H32">
-        <v>22000</v>
+        <v>7000</v>
       </c>
       <c r="I32">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="J32">
         <v>0</v>
       </c>
       <c r="K32" t="str">
-        <v>บอร์ดควบคุม PLC รองรับการเชื่อมต่อเครือข่าย Ethernet IP (PO: 2607001)</v>
+        <v>ตู้แร็คศูนย์คอมพิวเตอร์และเซิร์ฟเวอร์ Rack PC Center (PO: 2607001)</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>prod-pnp-sub-plc</v>
+        <v>prod-pnp-plc-dc</v>
       </c>
       <c r="B33" t="str">
-        <v>PLC-SUB-001</v>
+        <v>PLC-DC-001</v>
       </c>
       <c r="C33" t="str">
-        <v>Sub PLC Box + Aceessories</v>
+        <v>PLC Data Center Line</v>
       </c>
       <c r="D33" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E33" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>SOFTWARE</v>
       </c>
       <c r="F33" t="str">
         <v>EA</v>
       </c>
       <c r="G33">
-        <v>26000</v>
+        <v>150000</v>
       </c>
       <c r="H33">
-        <v>15000</v>
+        <v>80000</v>
       </c>
       <c r="I33">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J33">
         <v>0</v>
       </c>
       <c r="K33" t="str">
-        <v>ตู้ Sub PLC พร้อมอุปกรณ์ส่วนควบ Accessories (PO: 2607001)</v>
+        <v>ระบบศูนย์รวมและประมวลผลข้อมูลสายการผลิต PLC Data Center Line (PO: 2607001)</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>prod-pnp-rack-pc</v>
+        <v>prod-pnp-struct-sup</v>
       </c>
       <c r="B34" t="str">
-        <v>PC-RACK-001</v>
+        <v>STR-SUP-001</v>
       </c>
       <c r="C34" t="str">
-        <v>Rack PC Center</v>
+        <v>Stucture Support</v>
       </c>
       <c r="D34" t="str">
         <v>PRODUCT</v>
@@ -1881,10 +1843,10 @@
         <v>EA</v>
       </c>
       <c r="G34">
-        <v>12000</v>
+        <v>20000</v>
       </c>
       <c r="H34">
-        <v>7000</v>
+        <v>10000</v>
       </c>
       <c r="I34">
         <v>1</v>
@@ -1893,33 +1855,33 @@
         <v>0</v>
       </c>
       <c r="K34" t="str">
-        <v>ตู้แร็คศูนย์คอมพิวเตอร์และเซิร์ฟเวอร์ Rack PC Center (PO: 2607001)</v>
+        <v>ชุดโครงสร้างรองรับและฐานยึดอุปกรณ์ Structure Support (PO: 2607001)</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>prod-pnp-plc-dc</v>
+        <v>prod-pnp-pc-center</v>
       </c>
       <c r="B35" t="str">
-        <v>PLC-DC-001</v>
+        <v>PC-CTR-001</v>
       </c>
       <c r="C35" t="str">
-        <v>PLC Data Center Line</v>
+        <v>PC Center</v>
       </c>
       <c r="D35" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E35" t="str">
-        <v>SOFTWARE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F35" t="str">
         <v>EA</v>
       </c>
       <c r="G35">
-        <v>150000</v>
+        <v>123000</v>
       </c>
       <c r="H35">
-        <v>80000</v>
+        <v>75000</v>
       </c>
       <c r="I35">
         <v>1</v>
@@ -1928,33 +1890,33 @@
         <v>0</v>
       </c>
       <c r="K35" t="str">
-        <v>ระบบศูนย์รวมและประมวลผลข้อมูลสายการผลิต PLC Data Center Line (PO: 2607001)</v>
+        <v>เครื่องคอมพิวเตอร์แม่ข่ายประมวลผล PC Center (PO: 2607001)</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>prod-pnp-struct-sup</v>
+        <v>prod-pnp-pm-2607</v>
       </c>
       <c r="B36" t="str">
-        <v>STR-SUP-001</v>
+        <v>PNP-PM-2607</v>
       </c>
       <c r="C36" t="str">
-        <v>Stucture Support</v>
+        <v>Project Management (PO: 2607001)</v>
       </c>
       <c r="D36" t="str">
-        <v>PRODUCT</v>
+        <v>SERVICE</v>
       </c>
       <c r="E36" t="str">
-        <v>AUTOMATION_HARDWARE</v>
+        <v>ENGINEERING_SERVICE</v>
       </c>
       <c r="F36" t="str">
         <v>EA</v>
       </c>
       <c r="G36">
-        <v>20000</v>
+        <v>573552</v>
       </c>
       <c r="H36">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="I36">
         <v>1</v>
@@ -1963,18 +1925,18 @@
         <v>0</v>
       </c>
       <c r="K36" t="str">
-        <v>ชุดโครงสร้างรองรับและฐานยึดอุปกรณ์ Structure Support (PO: 2607001)</v>
+        <v>ค่าบริหารจัดการโครงการ ควบคุมงาน และทดสอบระบบ (PO: 2607001)</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>prod-pnp-pc-center</v>
+        <v>prod-spindle-01</v>
       </c>
       <c r="B37" t="str">
-        <v>PC-CTR-001</v>
+        <v>SPINDLE-ROLL-01</v>
       </c>
       <c r="C37" t="str">
-        <v>PC Center</v>
+        <v>Roller Paper Printer Spindle (แกนหมุนกระดาษเครื่องพิมพ์อัปเกรด)</v>
       </c>
       <c r="D37" t="str">
         <v>PRODUCT</v>
@@ -1983,57 +1945,57 @@
         <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F37" t="str">
-        <v>EA</v>
+        <v>Set</v>
       </c>
       <c r="G37">
-        <v>123000</v>
+        <v>1100</v>
       </c>
       <c r="H37">
-        <v>75000</v>
+        <v>1100</v>
       </c>
       <c r="I37">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="J37">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K37" t="str">
-        <v>เครื่องคอมพิวเตอร์แม่ข่ายประมวลผล PC Center (PO: 2607001)</v>
+        <v>แกนหมุนกระดาษเครื่องพิมพ์อัปเกรด (Roller Paper Printer Spindle)</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>prod-pnp-pm-2607</v>
+        <v>prod-box-minijb01</v>
       </c>
       <c r="B38" t="str">
-        <v>PNP-PM-2607</v>
+        <v>BOX-MINI-JB01</v>
       </c>
       <c r="C38" t="str">
-        <v>Project Management (PO: 2607001)</v>
+        <v>mini junction box</v>
       </c>
       <c r="D38" t="str">
-        <v>SERVICE</v>
+        <v>PRODUCT</v>
       </c>
       <c r="E38" t="str">
-        <v>ENGINEERING_SERVICE</v>
+        <v>AUTOMATION_HARDWARE</v>
       </c>
       <c r="F38" t="str">
-        <v>EA</v>
+        <v>Set</v>
       </c>
       <c r="G38">
-        <v>573552</v>
+        <v>300</v>
       </c>
       <c r="H38">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="I38">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="J38">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K38" t="str">
-        <v>ค่าบริหารจัดการโครงการ ควบคุมงาน และทดสอบระบบ (PO: 2607001)</v>
+        <v>mini junction box</v>
       </c>
     </row>
   </sheetData>
@@ -2045,7 +2007,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P26"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2714,34 +2676,34 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>doc-po-001</v>
+        <v>doc-tsf-qt-252155</v>
       </c>
       <c r="B17" t="str">
-        <v>PURCHASE_ORDER</v>
+        <v>QUOTATION</v>
       </c>
       <c r="C17" t="str">
-        <v>PO-202607-001</v>
+        <v>QT-2512-2155</v>
       </c>
       <c r="D17" t="str">
-        <v>2026-07-20</v>
+        <v>2025-12-24</v>
       </c>
       <c r="E17" t="str">
-        <v>2026-08-05</v>
+        <v>2026-01-23</v>
       </c>
       <c r="I17">
-        <v>132000</v>
+        <v>3645600</v>
       </c>
       <c r="J17">
-        <v>9240</v>
+        <v>248192</v>
       </c>
       <c r="K17">
-        <v>141240</v>
+        <v>3793792</v>
       </c>
       <c r="L17">
         <v>0</v>
       </c>
       <c r="M17">
-        <v>141240</v>
+        <v>3793792</v>
       </c>
       <c r="N17" t="str">
         <v>APPROVED</v>
@@ -2750,39 +2712,39 @@
         <v/>
       </c>
       <c r="P17" t="str">
-        <v>จัดส่งที่คลังสินค้า สมุทรปราการ</v>
+        <v>โครงการ TSF1 Auto pack LM1 (TSF1-LM1_Auto pack machine - K.Alongkorn) ตามใบสั่งซื้อ PO: PO252155 (Ref: CAP250095/) เงื่อนไขชำระเงิน 3 งวด: 1. 40% Down [฿1,517,516.80], 2. 30% After Process Work [฿1,138,137.60], 3. 30% After Complete Work [฿1,138,137.60] รับประกัน 1 ปี</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>doc-tsf-qt-252155</v>
+        <v>doc-pnp-qt-2505004</v>
       </c>
       <c r="B18" t="str">
         <v>QUOTATION</v>
       </c>
       <c r="C18" t="str">
-        <v>QT-2512-2155</v>
+        <v>QT-2505-004</v>
       </c>
       <c r="D18" t="str">
-        <v>2025-12-24</v>
+        <v>2025-05-07</v>
       </c>
       <c r="E18" t="str">
-        <v>2026-01-23</v>
+        <v>2025-06-06</v>
       </c>
       <c r="I18">
-        <v>3645600</v>
+        <v>4342990.38</v>
       </c>
       <c r="J18">
-        <v>248192</v>
+        <v>304009.33</v>
       </c>
       <c r="K18">
-        <v>3793792</v>
+        <v>4646999.71</v>
       </c>
       <c r="L18">
         <v>0</v>
       </c>
       <c r="M18">
-        <v>3793792</v>
+        <v>4646999.71</v>
       </c>
       <c r="N18" t="str">
         <v>APPROVED</v>
@@ -2791,39 +2753,39 @@
         <v/>
       </c>
       <c r="P18" t="str">
-        <v>โครงการ TSF1 Auto pack LM1 (TSF1-LM1_Auto pack machine - K.Alongkorn) ตามใบสั่งซื้อ PO: PO252155 (Ref: CAP250095/) เงื่อนไขชำระเงิน 3 งวด: 1. 40% Down [฿1,517,516.80], 2. 30% After Process Work [฿1,138,137.60], 3. 30% After Complete Work [฿1,138,137.60] รับประกัน 1 ปี</v>
+        <v>โครงการพัฒนาระบบ Traceability 5 ไลน์ผลิต (Fujipart Thailand Co., Ltd.) ตามใบสั่งซื้อลูกค้า PO: 2505004 ลงวันที่ 7 พ.ค. 2568 (เงื่อนไขชำระเงิน: ชำระเมื่อส่งของครบตามใบสั่งซื้อ, วางบิลวันที่ 1-25 ของทุกเดือน, ใบกำกับภาษี + สำเนา 5 ใบ)</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>doc-pnp-qt-2505004</v>
+        <v>doc-pnp-qt-2605001</v>
       </c>
       <c r="B19" t="str">
         <v>QUOTATION</v>
       </c>
       <c r="C19" t="str">
-        <v>QT-2505-004</v>
+        <v>QT-2605-001</v>
       </c>
       <c r="D19" t="str">
-        <v>2025-05-07</v>
+        <v>2026-05-02</v>
       </c>
       <c r="E19" t="str">
-        <v>2025-06-06</v>
+        <v>2026-06-01</v>
       </c>
       <c r="I19">
-        <v>4342990.38</v>
+        <v>2411500</v>
       </c>
       <c r="J19">
-        <v>304009.33</v>
+        <v>168805</v>
       </c>
       <c r="K19">
-        <v>4646999.71</v>
+        <v>2580305</v>
       </c>
       <c r="L19">
         <v>0</v>
       </c>
       <c r="M19">
-        <v>4646999.71</v>
+        <v>2580305</v>
       </c>
       <c r="N19" t="str">
         <v>APPROVED</v>
@@ -2832,18 +2794,18 @@
         <v/>
       </c>
       <c r="P19" t="str">
-        <v>โครงการพัฒนาระบบ Traceability 5 ไลน์ผลิต (Fujipart Thailand Co., Ltd.) ตามใบสั่งซื้อลูกค้า PO: 2505004 ลงวันที่ 7 พ.ค. 2568 (เงื่อนไขชำระเงิน: ชำระเมื่อส่งของครบตามใบสั่งซื้อ, วางบิลวันที่ 1-25 ของทุกเดือน, ใบกำกับภาษี + สำเนา 5 ใบ)</v>
+        <v>โครงการ Zone 1-6 (Fujipart Thailand) ตามใบสั่งซื้อ PO: 2605001 ลงวันที่ 2 พ.ค. 2569 (เงื่อนไข: ชำระค่าสินค้าเมื่อส่งของครบตามใบสั่งซื้อ, วางบิลวันที่ 1-25 ของทุกเดือน, ใบกำกับภาษี + สำเนา 5 ใบ)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>doc-pnp-qt-2605001</v>
+        <v>doc-pnp-qt-2605002</v>
       </c>
       <c r="B20" t="str">
         <v>QUOTATION</v>
       </c>
       <c r="C20" t="str">
-        <v>QT-2605-001</v>
+        <v>QT-2605-002</v>
       </c>
       <c r="D20" t="str">
         <v>2026-05-02</v>
@@ -2852,19 +2814,19 @@
         <v>2026-06-01</v>
       </c>
       <c r="I20">
-        <v>2411500</v>
+        <v>1177800</v>
       </c>
       <c r="J20">
-        <v>168805</v>
+        <v>82446</v>
       </c>
       <c r="K20">
-        <v>2580305</v>
+        <v>1260246</v>
       </c>
       <c r="L20">
         <v>0</v>
       </c>
       <c r="M20">
-        <v>2580305</v>
+        <v>1260246</v>
       </c>
       <c r="N20" t="str">
         <v>APPROVED</v>
@@ -2873,121 +2835,121 @@
         <v/>
       </c>
       <c r="P20" t="str">
-        <v>โครงการ Zone 1-6 (Fujipart Thailand) ตามใบสั่งซื้อ PO: 2605001 ลงวันที่ 2 พ.ค. 2569 (เงื่อนไข: ชำระค่าสินค้าเมื่อส่งของครบตามใบสั่งซื้อ, วางบิลวันที่ 1-25 ของทุกเดือน, ใบกำกับภาษี + สำเนา 5 ใบ)</v>
+        <v>โครงการ Zone 7 (Fujipart Thailand) ตามใบสั่งซื้อ PO: 2605002 ลงวันที่ 2 พ.ค. 2569 (เงื่อนไข: ชำระค่าสินค้าเมื่อส่งของครบตามใบสั่งซื้อ, วางบิลวันที่ 1-25 ของทุกเดือน, ใบกำกับภาษี + สำเนา 5 ใบ)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>doc-pnp-qt-2605002</v>
+        <v>doc-pnp-rec-2605002-1</v>
       </c>
       <c r="B21" t="str">
-        <v>QUOTATION</v>
+        <v>RECEIPT</v>
       </c>
       <c r="C21" t="str">
-        <v>QT-2605-002</v>
+        <v>REC-2605-002/1</v>
       </c>
       <c r="D21" t="str">
-        <v>2026-05-02</v>
+        <v>2026-05-25</v>
       </c>
       <c r="E21" t="str">
-        <v>2026-06-01</v>
+        <v>2026-05-25</v>
       </c>
       <c r="I21">
-        <v>1177800</v>
+        <v>353340</v>
       </c>
       <c r="J21">
-        <v>82446</v>
+        <v>24733.8</v>
       </c>
       <c r="K21">
-        <v>1260246</v>
+        <v>378073.8</v>
       </c>
       <c r="L21">
         <v>0</v>
       </c>
       <c r="M21">
-        <v>1260246</v>
+        <v>378073.8</v>
       </c>
       <c r="N21" t="str">
-        <v>APPROVED</v>
+        <v>PAID</v>
       </c>
       <c r="O21" t="str">
         <v/>
       </c>
       <c r="P21" t="str">
-        <v>โครงการ Zone 7 (Fujipart Thailand) ตามใบสั่งซื้อ PO: 2605002 ลงวันที่ 2 พ.ค. 2569 (เงื่อนไข: ชำระค่าสินค้าเมื่อส่งของครบตามใบสั่งซื้อ, วางบิลวันที่ 1-25 ของทุกเดือน, ใบกำกับภาษี + สำเนา 5 ใบ)</v>
+        <v>รับชำระเงินงวดที่ 1 (30% Downpayment) โครงการ Zone 7 (Fujipart) ตามใบสั่งซื้อ PO: 2605002 โอนเข้าบัญชี KBANK บจก. วอร์สเกต</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>doc-pnp-rec-2605002-1</v>
+        <v>doc-pnp-qt-2607001</v>
       </c>
       <c r="B22" t="str">
-        <v>RECEIPT</v>
+        <v>QUOTATION</v>
       </c>
       <c r="C22" t="str">
-        <v>REC-2605-002/1</v>
+        <v>QT-2607-001</v>
       </c>
       <c r="D22" t="str">
-        <v>2026-05-25</v>
+        <v>2026-07-17</v>
       </c>
       <c r="E22" t="str">
-        <v>2026-05-25</v>
+        <v>2026-08-16</v>
       </c>
       <c r="I22">
-        <v>353340</v>
+        <v>2439832</v>
       </c>
       <c r="J22">
-        <v>24733.8</v>
+        <v>170788.24</v>
       </c>
       <c r="K22">
-        <v>378073.8</v>
+        <v>2610620.24</v>
       </c>
       <c r="L22">
         <v>0</v>
       </c>
       <c r="M22">
-        <v>378073.8</v>
+        <v>2610620.24</v>
       </c>
       <c r="N22" t="str">
-        <v>PAID</v>
+        <v>APPROVED</v>
       </c>
       <c r="O22" t="str">
         <v/>
       </c>
       <c r="P22" t="str">
-        <v>รับชำระเงินงวดที่ 1 (30% Downpayment) โครงการ Zone 7 (Fujipart) ตามใบสั่งซื้อ PO: 2605002 โอนเข้าบัญชี KBANK บจก. วอร์สเกต</v>
+        <v>โครงการตามใบสั่งซื้อ PO: 2607001 ลงวันที่ 17 ก.ค. 2569 (รวมส่วนลดพิเศษ ฿45,560.00, ชำระค่าสินค้าเมื่อส่งของครบตามใบสั่งซื้อ, วางบิลวันที่ 1-25 ของทุกเดือน, ใบกำกับภาษี + สำเนา 5 ใบ)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>doc-pnp-qt-2607001</v>
+        <v>doc-pnp-do-2607001</v>
       </c>
       <c r="B23" t="str">
-        <v>QUOTATION</v>
+        <v>DELIVERY_ORDER</v>
       </c>
       <c r="C23" t="str">
-        <v>QT-2607-001</v>
+        <v>DO-2608-001</v>
       </c>
       <c r="D23" t="str">
-        <v>2026-07-17</v>
+        <v>2026-08-20</v>
       </c>
       <c r="E23" t="str">
-        <v>2026-08-16</v>
+        <v>2026-08-20</v>
       </c>
       <c r="I23">
-        <v>2439832</v>
+        <v>1196840</v>
       </c>
       <c r="J23">
-        <v>170788.24</v>
+        <v>83778.8</v>
       </c>
       <c r="K23">
-        <v>2610620.24</v>
+        <v>1280618.8</v>
       </c>
       <c r="L23">
         <v>0</v>
       </c>
       <c r="M23">
-        <v>2610620.24</v>
+        <v>1280618.8</v>
       </c>
       <c r="N23" t="str">
         <v>APPROVED</v>
@@ -2996,24 +2958,24 @@
         <v/>
       </c>
       <c r="P23" t="str">
-        <v>โครงการตามใบสั่งซื้อ PO: 2607001 ลงวันที่ 17 ก.ค. 2569 (รวมส่วนลดพิเศษ ฿45,560.00, ชำระค่าสินค้าเมื่อส่งของครบตามใบสั่งซื้อ, วางบิลวันที่ 1-25 ของทุกเดือน, ใบกำกับภาษี + สำเนา 5 ใบ)</v>
+        <v>ใบส่งของชั่วคราว / ใบส่งสินค้า ตามใบสั่งซื้อ PO: 2607001 รายการ Part ที่จัดส่งของ Line ADC โครงการ PLC Control Board (Ethernet IP) เพื่อตรวจรับหน้างานโรงงานชลบุรี</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>doc-pnp-do-2607001</v>
+        <v>doc-pnp-inv-2607001</v>
       </c>
       <c r="B24" t="str">
-        <v>DELIVERY_ORDER</v>
+        <v>INVOICE</v>
       </c>
       <c r="C24" t="str">
-        <v>DO-2608-001</v>
+        <v>INV-2608-001</v>
       </c>
       <c r="D24" t="str">
         <v>2026-08-20</v>
       </c>
       <c r="E24" t="str">
-        <v>2026-08-20</v>
+        <v>2026-09-19</v>
       </c>
       <c r="I24">
         <v>1196840</v>
@@ -3031,24 +2993,24 @@
         <v>1280618.8</v>
       </c>
       <c r="N24" t="str">
-        <v>APPROVED</v>
+        <v>PENDING</v>
       </c>
       <c r="O24" t="str">
         <v/>
       </c>
       <c r="P24" t="str">
-        <v>ใบส่งของชั่วคราว / ใบส่งสินค้า ตามใบสั่งซื้อ PO: 2607001 รายการ Part ที่จัดส่งของ Line ADC โครงการ PLC Control Board (Ethernet IP) เพื่อตรวจรับหน้างานโรงงานชลบุรี</v>
+        <v>ใบแจ้งหนี้ / ใบวางบิล ตามใบสั่งซื้อ PO: 2607001 และใบส่งของชั่วคราว DO-2608-001 (เงื่อนไขการชำระเงิน: เครดิต 30 วัน ครบกำหนด 19 ก.ย. 2569 โอนเข้าบัญชี KBANK บจก. วอร์สเกต)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>doc-pnp-inv-2607001</v>
+        <v>doc-pnp-tax-2607001</v>
       </c>
       <c r="B25" t="str">
-        <v>INVOICE</v>
+        <v>TAX_INVOICE</v>
       </c>
       <c r="C25" t="str">
-        <v>INV-2608-001</v>
+        <v>TAX-2608-001</v>
       </c>
       <c r="D25" t="str">
         <v>2026-08-20</v>
@@ -3072,45 +3034,45 @@
         <v>1280618.8</v>
       </c>
       <c r="N25" t="str">
-        <v>PENDING</v>
+        <v>APPROVED</v>
       </c>
       <c r="O25" t="str">
         <v/>
       </c>
       <c r="P25" t="str">
-        <v>ใบแจ้งหนี้ / ใบวางบิล ตามใบสั่งซื้อ PO: 2607001 และใบส่งของชั่วคราว DO-2608-001 (เงื่อนไขการชำระเงิน: เครดิต 30 วัน ครบกำหนด 19 ก.ย. 2569 โอนเข้าบัญชี KBANK บจก. วอร์สเกต)</v>
+        <v>ใบกำกับภาษี ตามใบสั่งซื้อ PO: 2607001, ใบส่งของชั่วคราว DO-2608-001 และใบแจ้งหนี้ INV-2608-001 รายการ Part Line ADC โครงการ PLC Control Board (Ethernet IP)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>doc-pnp-tax-2607001</v>
+        <v>doc-po-ptech-260901</v>
       </c>
       <c r="B26" t="str">
-        <v>TAX_INVOICE</v>
+        <v>PURCHASE_ORDER</v>
       </c>
       <c r="C26" t="str">
-        <v>TAX-2608-001</v>
+        <v>PO-2609-001</v>
       </c>
       <c r="D26" t="str">
-        <v>2026-08-20</v>
+        <v>2026-09-24</v>
       </c>
       <c r="E26" t="str">
-        <v>2026-09-19</v>
+        <v>2026-10-24</v>
       </c>
       <c r="I26">
-        <v>1196840</v>
+        <v>9000</v>
       </c>
       <c r="J26">
-        <v>83778.8</v>
+        <v>630</v>
       </c>
       <c r="K26">
-        <v>1280618.8</v>
+        <v>9630</v>
       </c>
       <c r="L26">
         <v>0</v>
       </c>
       <c r="M26">
-        <v>1280618.8</v>
+        <v>9630</v>
       </c>
       <c r="N26" t="str">
         <v>APPROVED</v>
@@ -3119,60 +3081,19 @@
         <v/>
       </c>
       <c r="P26" t="str">
-        <v>ใบกำกับภาษี ตามใบสั่งซื้อ PO: 2607001, ใบส่งของชั่วคราว DO-2608-001 และใบแจ้งหนี้ INV-2608-001 รายการ Part Line ADC โครงการ PLC Control Board (Ethernet IP)</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>doc-po-ptech-260901</v>
-      </c>
-      <c r="B27" t="str">
-        <v>PURCHASE_ORDER</v>
-      </c>
-      <c r="C27" t="str">
-        <v>PO-2609-001</v>
-      </c>
-      <c r="D27" t="str">
-        <v>2026-09-24</v>
-      </c>
-      <c r="E27" t="str">
-        <v>2026-10-24</v>
-      </c>
-      <c r="I27">
-        <v>9000</v>
-      </c>
-      <c r="J27">
-        <v>630</v>
-      </c>
-      <c r="K27">
-        <v>9630</v>
-      </c>
-      <c r="L27">
-        <v>0</v>
-      </c>
-      <c r="M27">
-        <v>9630</v>
-      </c>
-      <c r="N27" t="str">
-        <v>APPROVED</v>
-      </c>
-      <c r="O27" t="str">
-        <v/>
-      </c>
-      <c r="P27" t="str">
         <v>จัดส่งที่: บริษัท วอร์สเกต จำกัด (สำนักงานใหญ่) หมู่บ้าน พฤกษาวิลล์ 46/1 เลขที่ 50/8 หมู่ 4 ตำบลคลองสาม อำเภอคลองหลวง จังหวัดปทุมธานี 12120 โทร. 083-066-7309</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P26"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L93"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4336,13 +4257,13 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>PO-202607-001</v>
+        <v>QT-2512-2155</v>
       </c>
       <c r="B44" t="str">
-        <v>PURCHASE_ORDER</v>
+        <v>QUOTATION</v>
       </c>
       <c r="C44" t="str">
-        <v>2026-07-20</v>
+        <v>2025-12-24</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -4351,13 +4272,13 @@
         <v/>
       </c>
       <c r="G44" t="str">
-        <v>สั่งซื้อเพื่อสต็อกโครงการใหม่</v>
+        <v>ชุดสถานีเรียงโฟมอัตโนมัติ (Station Stacker Foam) เครื่อง TSF1 Auto pack LM1 (ETA: 09/01/2026)</v>
       </c>
       <c r="H44">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I44" t="str">
-        <v>เครื่อง</v>
+        <v>SET</v>
       </c>
       <c r="K44">
         <v>0</v>
@@ -4374,13 +4295,13 @@
         <v>2025-12-24</v>
       </c>
       <c r="E45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F45" t="str">
         <v/>
       </c>
       <c r="G45" t="str">
-        <v>ชุดสถานีเรียงโฟมอัตโนมัติ (Station Stacker Foam) เครื่อง TSF1 Auto pack LM1 (ETA: 09/01/2026)</v>
+        <v>ชุดสถานีเปิดถุงและบรรจุโฟม (Station Open Bag &amp; Insert Foam) (ETA: 09/01/2026)</v>
       </c>
       <c r="H45">
         <v>1</v>
@@ -4403,13 +4324,13 @@
         <v>2025-12-24</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F46" t="str">
         <v/>
       </c>
       <c r="G46" t="str">
-        <v>ชุดสถานีเปิดถุงและบรรจุโฟม (Station Open Bag &amp; Insert Foam) (ETA: 09/01/2026)</v>
+        <v>ชุดสถานีเรียงพาเลทโฟม (Station Pallet Stacker Foam) (ETA: 09/01/2026)</v>
       </c>
       <c r="H46">
         <v>1</v>
@@ -4432,13 +4353,13 @@
         <v>2025-12-24</v>
       </c>
       <c r="E47">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F47" t="str">
         <v/>
       </c>
       <c r="G47" t="str">
-        <v>ชุดสถานีเรียงพาเลทโฟม (Station Pallet Stacker Foam) (ETA: 09/01/2026)</v>
+        <v>ตู้ควบคุมระบบไฟฟ้าและ PLC (Control Box System) (ETA: 09/01/2026)</v>
       </c>
       <c r="H47">
         <v>1</v>
@@ -4461,19 +4382,19 @@
         <v>2025-12-24</v>
       </c>
       <c r="E48">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F48" t="str">
         <v/>
       </c>
       <c r="G48" t="str">
-        <v>ตู้ควบคุมระบบไฟฟ้าและ PLC (Control Box System) (ETA: 09/01/2026)</v>
+        <v>ค่าแรงวิศวกร ประกอบ ติดตั้ง และทดสอบระบบ (ETA: 09/01/2026)</v>
       </c>
       <c r="H48">
         <v>1</v>
       </c>
       <c r="I48" t="str">
-        <v>SET</v>
+        <v>JOB</v>
       </c>
       <c r="K48">
         <v>0</v>
@@ -4490,13 +4411,13 @@
         <v>2025-12-24</v>
       </c>
       <c r="E49">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F49" t="str">
         <v/>
       </c>
       <c r="G49" t="str">
-        <v>ค่าแรงวิศวกร ประกอบ ติดตั้ง และทดสอบระบบ (ETA: 09/01/2026)</v>
+        <v>ค่าขนส่งและที่พักเดินทางหน้างานโรงงานชลบุรี (ETA: 09/01/2026)</v>
       </c>
       <c r="H49">
         <v>1</v>
@@ -4519,13 +4440,13 @@
         <v>2025-12-24</v>
       </c>
       <c r="E50">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F50" t="str">
         <v/>
       </c>
       <c r="G50" t="str">
-        <v>ค่าขนส่งและที่พักเดินทางหน้างานโรงงานชลบุรี (ETA: 09/01/2026)</v>
+        <v>ค่าบริหารโครงการและรับประกันระบบ 1 ปี TSF1 Auto pack LM1 (ETA: 09/01/2026)</v>
       </c>
       <c r="H50">
         <v>1</v>
@@ -4539,28 +4460,28 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>QT-2512-2155</v>
+        <v>QT-2505-004</v>
       </c>
       <c r="B51" t="str">
         <v>QUOTATION</v>
       </c>
       <c r="C51" t="str">
-        <v>2025-12-24</v>
+        <v>2025-05-07</v>
       </c>
       <c r="E51">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F51" t="str">
         <v/>
       </c>
       <c r="G51" t="str">
-        <v>ค่าบริหารโครงการและรับประกันระบบ 1 ปี TSF1 Auto pack LM1 (ETA: 09/01/2026)</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Corrugating Line โครงการ Fujipart (Thailand) Co., Ltd.</v>
       </c>
       <c r="H51">
         <v>1</v>
       </c>
       <c r="I51" t="str">
-        <v>JOB</v>
+        <v>Job</v>
       </c>
       <c r="K51">
         <v>0</v>
@@ -4577,13 +4498,13 @@
         <v>2025-05-07</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F52" t="str">
         <v/>
       </c>
       <c r="G52" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Corrugating Line โครงการ Fujipart (Thailand) Co., Ltd.</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Winding Line โครงการ Fujipart (Thailand) Co., Ltd.</v>
       </c>
       <c r="H52">
         <v>1</v>
@@ -4606,13 +4527,13 @@
         <v>2025-05-07</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F53" t="str">
         <v/>
       </c>
       <c r="G53" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Winding Line โครงการ Fujipart (Thailand) Co., Ltd.</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Adhesive &amp; Spin Winding Line โครงการ Fujipart (Thailand) Co., Ltd.</v>
       </c>
       <c r="H53">
         <v>1</v>
@@ -4635,13 +4556,13 @@
         <v>2025-05-07</v>
       </c>
       <c r="E54">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F54" t="str">
         <v/>
       </c>
       <c r="G54" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Adhesive &amp; Spin Winding Line โครงการ Fujipart (Thailand) Co., Ltd.</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต DF4 Line โครงการ Fujipart (Thailand) Co., Ltd.</v>
       </c>
       <c r="H54">
         <v>1</v>
@@ -4664,13 +4585,13 @@
         <v>2025-05-07</v>
       </c>
       <c r="E55">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F55" t="str">
         <v/>
       </c>
       <c r="G55" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต DF4 Line โครงการ Fujipart (Thailand) Co., Ltd.</v>
+        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Packing Line โครงการ Fujipart (Thailand) Co., Ltd.</v>
       </c>
       <c r="H55">
         <v>1</v>
@@ -4684,28 +4605,28 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>QT-2505-004</v>
+        <v>QT-2605-001</v>
       </c>
       <c r="B56" t="str">
         <v>QUOTATION</v>
       </c>
       <c r="C56" t="str">
-        <v>2025-05-07</v>
+        <v>2026-05-02</v>
       </c>
       <c r="E56">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F56" t="str">
         <v/>
       </c>
       <c r="G56" t="str">
-        <v>ระบบซอฟต์แวร์ตรวจสอบย้อนกลับไลน์ผลิต Packing Line โครงการ Fujipart (Thailand) Co., Ltd.</v>
+        <v>ชุดชิ้นงานโครงสร้างและประกอบมาตรฐาน (Zone 1-6) โครงการ Fujipart (Thailand) Co., Ltd.</v>
       </c>
       <c r="H56">
         <v>1</v>
       </c>
       <c r="I56" t="str">
-        <v>Job</v>
+        <v>Set</v>
       </c>
       <c r="K56">
         <v>0</v>
@@ -4722,19 +4643,19 @@
         <v>2026-05-02</v>
       </c>
       <c r="E57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F57" t="str">
         <v/>
       </c>
       <c r="G57" t="str">
-        <v>ชุดชิ้นงานโครงสร้างและประกอบมาตรฐาน (Zone 1-6) โครงการ Fujipart (Thailand) Co., Ltd.</v>
+        <v>ค่าแรงประกอบ ติดตั้ง และทดสอบระบบ (Zone 1-6)</v>
       </c>
       <c r="H57">
         <v>1</v>
       </c>
       <c r="I57" t="str">
-        <v>Set</v>
+        <v>Job</v>
       </c>
       <c r="K57">
         <v>0</v>
@@ -4751,19 +4672,19 @@
         <v>2026-05-02</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F58" t="str">
         <v/>
       </c>
       <c r="G58" t="str">
-        <v>ค่าแรงประกอบ ติดตั้ง และทดสอบระบบ (Zone 1-6)</v>
+        <v>ค่าขนส่งและที่พักเดินทางหน้างานโรงงานชลบุรี (Zone 1-6)</v>
       </c>
       <c r="H58">
         <v>1</v>
       </c>
       <c r="I58" t="str">
-        <v>Job</v>
+        <v>EA</v>
       </c>
       <c r="K58">
         <v>0</v>
@@ -4780,13 +4701,13 @@
         <v>2026-05-02</v>
       </c>
       <c r="E59">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F59" t="str">
         <v/>
       </c>
       <c r="G59" t="str">
-        <v>ค่าขนส่งและที่พักเดินทางหน้างานโรงงานชลบุรี (Zone 1-6)</v>
+        <v>ค่าบริหารโครงการ ควบคุมงาน และทดสอบระบบ Zone 1-6</v>
       </c>
       <c r="H59">
         <v>1</v>
@@ -4800,7 +4721,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>QT-2605-001</v>
+        <v>QT-2605-002</v>
       </c>
       <c r="B60" t="str">
         <v>QUOTATION</v>
@@ -4809,19 +4730,19 @@
         <v>2026-05-02</v>
       </c>
       <c r="E60">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F60" t="str">
         <v/>
       </c>
       <c r="G60" t="str">
-        <v>ค่าบริหารโครงการ ควบคุมงาน และทดสอบระบบ Zone 1-6</v>
+        <v>ชุดชิ้นงานโครงสร้างและประกอบมาตรฐาน (Zone 7) โครงการ Fujipart (Thailand) Co., Ltd.</v>
       </c>
       <c r="H60">
         <v>1</v>
       </c>
       <c r="I60" t="str">
-        <v>EA</v>
+        <v>Set</v>
       </c>
       <c r="K60">
         <v>0</v>
@@ -4838,19 +4759,19 @@
         <v>2026-05-02</v>
       </c>
       <c r="E61">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" t="str">
         <v/>
       </c>
       <c r="G61" t="str">
-        <v>ชุดชิ้นงานโครงสร้างและประกอบมาตรฐาน (Zone 7) โครงการ Fujipart (Thailand) Co., Ltd.</v>
+        <v>ค่าแรงประกอบ ติดตั้ง และทดสอบระบบ (Zone 7)</v>
       </c>
       <c r="H61">
         <v>1</v>
       </c>
       <c r="I61" t="str">
-        <v>Set</v>
+        <v>Job</v>
       </c>
       <c r="K61">
         <v>0</v>
@@ -4867,19 +4788,19 @@
         <v>2026-05-02</v>
       </c>
       <c r="E62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F62" t="str">
         <v/>
       </c>
       <c r="G62" t="str">
-        <v>ค่าแรงประกอบ ติดตั้ง และทดสอบระบบ (Zone 7)</v>
+        <v>ค่าขนส่งและที่พักเดินทางหน้างานโรงงานชลบุรี (Zone 7)</v>
       </c>
       <c r="H62">
         <v>1</v>
       </c>
       <c r="I62" t="str">
-        <v>Job</v>
+        <v>EA</v>
       </c>
       <c r="K62">
         <v>0</v>
@@ -4896,13 +4817,13 @@
         <v>2026-05-02</v>
       </c>
       <c r="E63">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F63" t="str">
         <v/>
       </c>
       <c r="G63" t="str">
-        <v>ค่าขนส่งและที่พักเดินทางหน้างานโรงงานชลบุรี (Zone 7)</v>
+        <v>ค่าบริหารโครงการ ควบคุมงาน และทดสอบระบบ Zone 7</v>
       </c>
       <c r="H63">
         <v>1</v>
@@ -4916,28 +4837,28 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>QT-2605-002</v>
+        <v>REC-2605-002/1</v>
       </c>
       <c r="B64" t="str">
-        <v>QUOTATION</v>
+        <v>RECEIPT</v>
       </c>
       <c r="C64" t="str">
-        <v>2026-05-02</v>
+        <v>2026-05-25</v>
       </c>
       <c r="E64">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F64" t="str">
         <v/>
       </c>
       <c r="G64" t="str">
-        <v>ค่าบริหารโครงการ ควบคุมงาน และทดสอบระบบ Zone 7</v>
+        <v>โครงการ Zone 7 (Fujipart Thailand) ตามใบสั่งซื้อ PO: 2605002 และใบแจ้งหนี้ INV-2605-002/1</v>
       </c>
       <c r="H64">
         <v>1</v>
       </c>
       <c r="I64" t="str">
-        <v>EA</v>
+        <v>งวด</v>
       </c>
       <c r="K64">
         <v>0</v>
@@ -4945,13 +4866,13 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>REC-2605-002/1</v>
+        <v>QT-2607-001</v>
       </c>
       <c r="B65" t="str">
-        <v>RECEIPT</v>
+        <v>QUOTATION</v>
       </c>
       <c r="C65" t="str">
-        <v>2026-05-25</v>
+        <v>2026-07-17</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -4960,13 +4881,13 @@
         <v/>
       </c>
       <c r="G65" t="str">
-        <v>โครงการ Zone 7 (Fujipart Thailand) ตามใบสั่งซื้อ PO: 2605002 และใบแจ้งหนี้ INV-2605-002/1</v>
+        <v>ชุดบอร์ดควบคุม PLC รองรับการสื่อสารข้อมูลระบบ Ethernet IP</v>
       </c>
       <c r="H65">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="I65" t="str">
-        <v>งวด</v>
+        <v>EA</v>
       </c>
       <c r="K65">
         <v>0</v>
@@ -4983,16 +4904,16 @@
         <v>2026-07-17</v>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F66" t="str">
         <v/>
       </c>
       <c r="G66" t="str">
-        <v>ชุดบอร์ดควบคุม PLC รองรับการสื่อสารข้อมูลระบบ Ethernet IP</v>
+        <v>ตู้ Sub PLC พร้อมอุปกรณ์ส่วนควบและเดินสายไฟสัญญาณ</v>
       </c>
       <c r="H66">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="I66" t="str">
         <v>EA</v>
@@ -5012,16 +4933,16 @@
         <v>2026-07-17</v>
       </c>
       <c r="E67">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F67" t="str">
         <v/>
       </c>
       <c r="G67" t="str">
-        <v>ตู้ Sub PLC พร้อมอุปกรณ์ส่วนควบและเดินสายไฟสัญญาณ</v>
+        <v>ตู้แร็คระบบศูนย์คอมพิวเตอร์ Rack PC Center</v>
       </c>
       <c r="H67">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I67" t="str">
         <v>EA</v>
@@ -5041,13 +4962,13 @@
         <v>2026-07-17</v>
       </c>
       <c r="E68">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F68" t="str">
         <v/>
       </c>
       <c r="G68" t="str">
-        <v>ตู้แร็คระบบศูนย์คอมพิวเตอร์ Rack PC Center</v>
+        <v>ระบบศูนย์รวมและเชื่อมต่อข้อมูลสายการผลิต PLC Data Center Line</v>
       </c>
       <c r="H68">
         <v>1</v>
@@ -5070,13 +4991,13 @@
         <v>2026-07-17</v>
       </c>
       <c r="E69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F69" t="str">
         <v/>
       </c>
       <c r="G69" t="str">
-        <v>ระบบศูนย์รวมและเชื่อมต่อข้อมูลสายการผลิต PLC Data Center Line</v>
+        <v>ชุดโครงสร้างรองรับและฐานยึดอุปกรณ์ Structure Support</v>
       </c>
       <c r="H69">
         <v>1</v>
@@ -5099,13 +5020,13 @@
         <v>2026-07-17</v>
       </c>
       <c r="E70">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F70" t="str">
         <v/>
       </c>
       <c r="G70" t="str">
-        <v>ชุดโครงสร้างรองรับและฐานยึดอุปกรณ์ Structure Support</v>
+        <v>เครื่องคอมพิวเตอร์แม่ข่ายประมวลผล PC Center</v>
       </c>
       <c r="H70">
         <v>1</v>
@@ -5128,19 +5049,19 @@
         <v>2026-07-17</v>
       </c>
       <c r="E71">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F71" t="str">
         <v/>
       </c>
       <c r="G71" t="str">
-        <v>เครื่องคอมพิวเตอร์แม่ข่ายประมวลผล PC Center</v>
+        <v>ค่าแรงวิศวกรและทีมช่างประกอบ ติดตั้ง และทดสอบระบบ</v>
       </c>
       <c r="H71">
         <v>1</v>
       </c>
       <c r="I71" t="str">
-        <v>EA</v>
+        <v>Job</v>
       </c>
       <c r="K71">
         <v>0</v>
@@ -5157,19 +5078,19 @@
         <v>2026-07-17</v>
       </c>
       <c r="E72">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F72" t="str">
         <v/>
       </c>
       <c r="G72" t="str">
-        <v>ค่าแรงวิศวกรและทีมช่างประกอบ ติดตั้ง และทดสอบระบบ</v>
+        <v>ค่าขนส่งและที่พักเดินทางหน้างานโรงงานชลบุรี</v>
       </c>
       <c r="H72">
         <v>1</v>
       </c>
       <c r="I72" t="str">
-        <v>Job</v>
+        <v>EA</v>
       </c>
       <c r="K72">
         <v>0</v>
@@ -5186,13 +5107,13 @@
         <v>2026-07-17</v>
       </c>
       <c r="E73">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F73" t="str">
         <v/>
       </c>
       <c r="G73" t="str">
-        <v>ค่าขนส่งและที่พักเดินทางหน้างานโรงงานชลบุรี</v>
+        <v>ค่าบริหารโครงการ ควบคุมงาน และทดสอบระบบ</v>
       </c>
       <c r="H73">
         <v>1</v>
@@ -5206,25 +5127,25 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>QT-2607-001</v>
+        <v>DO-2608-001</v>
       </c>
       <c r="B74" t="str">
-        <v>QUOTATION</v>
+        <v>DELIVERY_ORDER</v>
       </c>
       <c r="C74" t="str">
-        <v>2026-07-17</v>
+        <v>2026-08-20</v>
       </c>
       <c r="E74">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F74" t="str">
         <v/>
       </c>
       <c r="G74" t="str">
-        <v>ค่าบริหารโครงการ ควบคุมงาน และทดสอบระบบ</v>
+        <v>Part: CJ1W-EIP21 | Brand: OMRON (Line ADC)</v>
       </c>
       <c r="H74">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="I74" t="str">
         <v>EA</v>
@@ -5233,7 +5154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" xml:space="preserve">
       <c r="A75" t="str">
         <v>DO-2608-001</v>
       </c>
@@ -5244,52 +5165,54 @@
         <v>2026-08-20</v>
       </c>
       <c r="E75">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F75" t="str">
         <v/>
       </c>
-      <c r="G75" t="str">
-        <v>Part: CJ1W-EIP21 | Brand: OMRON (Line ADC)</v>
-      </c>
-      <c r="H75">
-        <v>21</v>
-      </c>
-      <c r="I75" t="str">
-        <v>EA</v>
-      </c>
-      <c r="K75">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" xml:space="preserve">
-      <c r="A76" t="str">
-        <v>DO-2608-001</v>
-      </c>
-      <c r="B76" t="str">
-        <v>DELIVERY_ORDER</v>
-      </c>
-      <c r="C76" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="E76">
-        <v>2</v>
-      </c>
-      <c r="F76" t="str">
-        <v/>
-      </c>
-      <c r="G76" t="str" xml:space="preserve">
+      <c r="G75" t="str" xml:space="preserve">
         <v xml:space="preserve">ประกอบด้วย:
 • 2.1 PLC POWER SUPPLY UNIT (CJ1W-PA202 OMRON) 6 EA
 • 2.2 MODULE LINK RACK UNIT (CJ1W-IC101 OMRON) 6 EA
 • 2.3 MODULE LINK RACK UNIT (CJ1W-II101 OMRON) 6 EA
 • 2.4 CABLE LINK RACK (CS1W-CN223 2M OMRON) 6 EA</v>
       </c>
+      <c r="H75">
+        <v>6</v>
+      </c>
+      <c r="I75" t="str">
+        <v>SET</v>
+      </c>
+      <c r="K75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" xml:space="preserve">
+      <c r="A76" t="str">
+        <v>DO-2608-001</v>
+      </c>
+      <c r="B76" t="str">
+        <v>DELIVERY_ORDER</v>
+      </c>
+      <c r="C76" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="E76">
+        <v>3</v>
+      </c>
+      <c r="F76" t="str">
+        <v/>
+      </c>
+      <c r="G76" t="str" xml:space="preserve">
+        <v xml:space="preserve">ประกอบด้วย:
+• 3.1 SWITCHING HUB (CBS110-24T-EU CISCO) 1 EA
+• 3.2 ตู้เซิร์ฟเวอร์เครือข่าย 12U (ACR-12U-W APOLLO) 1 EA</v>
+      </c>
       <c r="H76">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I76" t="str">
-        <v>SET</v>
+        <v>EA</v>
       </c>
       <c r="K76">
         <v>0</v>
@@ -5306,43 +5229,12 @@
         <v>2026-08-20</v>
       </c>
       <c r="E77">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F77" t="str">
         <v/>
       </c>
       <c r="G77" t="str" xml:space="preserve">
-        <v xml:space="preserve">ประกอบด้วย:
-• 3.1 SWITCHING HUB (CBS110-24T-EU CISCO) 1 EA
-• 3.2 ตู้เซิร์ฟเวอร์เครือข่าย 12U (ACR-12U-W APOLLO) 1 EA</v>
-      </c>
-      <c r="H77">
-        <v>1</v>
-      </c>
-      <c r="I77" t="str">
-        <v>EA</v>
-      </c>
-      <c r="K77">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" xml:space="preserve">
-      <c r="A78" t="str">
-        <v>DO-2608-001</v>
-      </c>
-      <c r="B78" t="str">
-        <v>DELIVERY_ORDER</v>
-      </c>
-      <c r="C78" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="E78">
-        <v>4</v>
-      </c>
-      <c r="F78" t="str">
-        <v/>
-      </c>
-      <c r="G78" t="str" xml:space="preserve">
         <v xml:space="preserve">ประกอบด้วย:
 • 4.1 BOX CONTROL (CE-01 TEMCO) 1 EA
 • 4.2 POWER SUPPLY PLC (CJ1W-PA202 OMRON) 1 EA
@@ -5350,6 +5242,36 @@
 • 4.4 INPUT MODULE (CJ1W-211 OMRON) 1 EA
 • 4.5 CIRCUIT PROTECTION (CP30-B 5A FUJI) 1 EA</v>
       </c>
+      <c r="H77">
+        <v>1</v>
+      </c>
+      <c r="I77" t="str">
+        <v>SET</v>
+      </c>
+      <c r="K77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" xml:space="preserve">
+      <c r="A78" t="str">
+        <v>DO-2608-001</v>
+      </c>
+      <c r="B78" t="str">
+        <v>DELIVERY_ORDER</v>
+      </c>
+      <c r="C78" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="E78">
+        <v>5</v>
+      </c>
+      <c r="F78" t="str">
+        <v/>
+      </c>
+      <c r="G78" t="str" xml:space="preserve">
+        <v xml:space="preserve">ประกอบด้วย:
+• 5.1 Aluminium profile (LOCAL) 1 SET</v>
+      </c>
       <c r="H78">
         <v>1</v>
       </c>
@@ -5371,58 +5293,57 @@
         <v>2026-08-20</v>
       </c>
       <c r="E79">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F79" t="str">
         <v/>
       </c>
       <c r="G79" t="str" xml:space="preserve">
-        <v xml:space="preserve">ประกอบด้วย:
-• 5.1 Aluminium profile (LOCAL) 1 SET</v>
-      </c>
-      <c r="H79">
-        <v>1</v>
-      </c>
-      <c r="I79" t="str">
-        <v>SET</v>
-      </c>
-      <c r="K79">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" xml:space="preserve">
-      <c r="A80" t="str">
-        <v>DO-2608-001</v>
-      </c>
-      <c r="B80" t="str">
-        <v>DELIVERY_ORDER</v>
-      </c>
-      <c r="C80" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="E80">
-        <v>6</v>
-      </c>
-      <c r="F80" t="str">
-        <v/>
-      </c>
-      <c r="G80" t="str" xml:space="preserve">
         <v xml:space="preserve">ประกอบด้วย:
 • 6.1 คอมพิวเตอร์ประกอบ (WG-93342286-SO26008123) 1 SET
 • 6.2 เครื่องสำรองไฟ UPS (ZIRCON AX 1000VA/550W) 1 EA
 • 6.3 MOUSE + KEYBOARD (MK120 CORDED LOGITECH) 1 EA</v>
       </c>
+      <c r="H79">
+        <v>1</v>
+      </c>
+      <c r="I79" t="str">
+        <v>SET</v>
+      </c>
+      <c r="K79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>INV-2608-001</v>
+      </c>
+      <c r="B80" t="str">
+        <v>INVOICE</v>
+      </c>
+      <c r="C80" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="E80">
+        <v>1</v>
+      </c>
+      <c r="F80" t="str">
+        <v/>
+      </c>
+      <c r="G80" t="str">
+        <v>Part: CJ1W-EIP21 | Brand: OMRON (Line ADC)</v>
+      </c>
       <c r="H80">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="I80" t="str">
-        <v>SET</v>
+        <v>EA</v>
       </c>
       <c r="K80">
         <v>0</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" xml:space="preserve">
       <c r="A81" t="str">
         <v>INV-2608-001</v>
       </c>
@@ -5433,52 +5354,54 @@
         <v>2026-08-20</v>
       </c>
       <c r="E81">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F81" t="str">
         <v/>
       </c>
-      <c r="G81" t="str">
-        <v>Part: CJ1W-EIP21 | Brand: OMRON (Line ADC)</v>
-      </c>
-      <c r="H81">
-        <v>21</v>
-      </c>
-      <c r="I81" t="str">
-        <v>EA</v>
-      </c>
-      <c r="K81">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" xml:space="preserve">
-      <c r="A82" t="str">
-        <v>INV-2608-001</v>
-      </c>
-      <c r="B82" t="str">
-        <v>INVOICE</v>
-      </c>
-      <c r="C82" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="E82">
-        <v>2</v>
-      </c>
-      <c r="F82" t="str">
-        <v/>
-      </c>
-      <c r="G82" t="str" xml:space="preserve">
+      <c r="G81" t="str" xml:space="preserve">
         <v xml:space="preserve">ประกอบด้วย:
 • 2.1 PLC POWER SUPPLY UNIT (CJ1W-PA202 OMRON) 6 EA
 • 2.2 MODULE LINK RACK UNIT (CJ1W-IC101 OMRON) 6 EA
 • 2.3 MODULE LINK RACK UNIT (CJ1W-II101 OMRON) 6 EA
 • 2.4 CABLE LINK RACK (CS1W-CN223 2M OMRON) 6 EA</v>
       </c>
+      <c r="H81">
+        <v>6</v>
+      </c>
+      <c r="I81" t="str">
+        <v>SET</v>
+      </c>
+      <c r="K81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" xml:space="preserve">
+      <c r="A82" t="str">
+        <v>INV-2608-001</v>
+      </c>
+      <c r="B82" t="str">
+        <v>INVOICE</v>
+      </c>
+      <c r="C82" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="E82">
+        <v>3</v>
+      </c>
+      <c r="F82" t="str">
+        <v/>
+      </c>
+      <c r="G82" t="str" xml:space="preserve">
+        <v xml:space="preserve">ประกอบด้วย:
+• 3.1 SWITCHING HUB (CBS110-24T-EU CISCO) 1 EA
+• 3.2 ตู้เซิร์ฟเวอร์เครือข่าย 12U (ACR-12U-W APOLLO) 1 EA</v>
+      </c>
       <c r="H82">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I82" t="str">
-        <v>SET</v>
+        <v>EA</v>
       </c>
       <c r="K82">
         <v>0</v>
@@ -5495,43 +5418,12 @@
         <v>2026-08-20</v>
       </c>
       <c r="E83">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F83" t="str">
         <v/>
       </c>
       <c r="G83" t="str" xml:space="preserve">
-        <v xml:space="preserve">ประกอบด้วย:
-• 3.1 SWITCHING HUB (CBS110-24T-EU CISCO) 1 EA
-• 3.2 ตู้เซิร์ฟเวอร์เครือข่าย 12U (ACR-12U-W APOLLO) 1 EA</v>
-      </c>
-      <c r="H83">
-        <v>1</v>
-      </c>
-      <c r="I83" t="str">
-        <v>EA</v>
-      </c>
-      <c r="K83">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" xml:space="preserve">
-      <c r="A84" t="str">
-        <v>INV-2608-001</v>
-      </c>
-      <c r="B84" t="str">
-        <v>INVOICE</v>
-      </c>
-      <c r="C84" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="E84">
-        <v>4</v>
-      </c>
-      <c r="F84" t="str">
-        <v/>
-      </c>
-      <c r="G84" t="str" xml:space="preserve">
         <v xml:space="preserve">ประกอบด้วย:
 • 4.1 BOX CONTROL (CE-01 TEMCO) 1 EA
 • 4.2 POWER SUPPLY PLC (CJ1W-PA202 OMRON) 1 EA
@@ -5539,6 +5431,36 @@
 • 4.4 INPUT MODULE (CJ1W-211 OMRON) 1 EA
 • 4.5 CIRCUIT PROTECTION (CP30-B 5A FUJI) 1 EA</v>
       </c>
+      <c r="H83">
+        <v>1</v>
+      </c>
+      <c r="I83" t="str">
+        <v>SET</v>
+      </c>
+      <c r="K83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" xml:space="preserve">
+      <c r="A84" t="str">
+        <v>INV-2608-001</v>
+      </c>
+      <c r="B84" t="str">
+        <v>INVOICE</v>
+      </c>
+      <c r="C84" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="E84">
+        <v>5</v>
+      </c>
+      <c r="F84" t="str">
+        <v/>
+      </c>
+      <c r="G84" t="str" xml:space="preserve">
+        <v xml:space="preserve">ประกอบด้วย:
+• 5.1 Aluminium profile (LOCAL) 1 SET</v>
+      </c>
       <c r="H84">
         <v>1</v>
       </c>
@@ -5560,58 +5482,57 @@
         <v>2026-08-20</v>
       </c>
       <c r="E85">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F85" t="str">
         <v/>
       </c>
       <c r="G85" t="str" xml:space="preserve">
-        <v xml:space="preserve">ประกอบด้วย:
-• 5.1 Aluminium profile (LOCAL) 1 SET</v>
-      </c>
-      <c r="H85">
-        <v>1</v>
-      </c>
-      <c r="I85" t="str">
-        <v>SET</v>
-      </c>
-      <c r="K85">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86" xml:space="preserve">
-      <c r="A86" t="str">
-        <v>INV-2608-001</v>
-      </c>
-      <c r="B86" t="str">
-        <v>INVOICE</v>
-      </c>
-      <c r="C86" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="E86">
-        <v>6</v>
-      </c>
-      <c r="F86" t="str">
-        <v/>
-      </c>
-      <c r="G86" t="str" xml:space="preserve">
         <v xml:space="preserve">ประกอบด้วย:
 • 6.1 คอมพิวเตอร์ประกอบ (WG-93342286-SO26008123) 1 SET
 • 6.2 เครื่องสำรองไฟ UPS (ZIRCON AX 1000VA/550W) 1 EA
 • 6.3 MOUSE + KEYBOARD (MK120 CORDED LOGITECH) 1 EA</v>
       </c>
+      <c r="H85">
+        <v>1</v>
+      </c>
+      <c r="I85" t="str">
+        <v>SET</v>
+      </c>
+      <c r="K85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>TAX-2608-001</v>
+      </c>
+      <c r="B86" t="str">
+        <v>TAX_INVOICE</v>
+      </c>
+      <c r="C86" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="E86">
+        <v>1</v>
+      </c>
+      <c r="F86" t="str">
+        <v/>
+      </c>
+      <c r="G86" t="str">
+        <v>Part: CJ1W-EIP21 | Brand: OMRON (Line ADC)</v>
+      </c>
       <c r="H86">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="I86" t="str">
-        <v>SET</v>
+        <v>EA</v>
       </c>
       <c r="K86">
         <v>0</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" xml:space="preserve">
       <c r="A87" t="str">
         <v>TAX-2608-001</v>
       </c>
@@ -5622,52 +5543,54 @@
         <v>2026-08-20</v>
       </c>
       <c r="E87">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F87" t="str">
         <v/>
       </c>
-      <c r="G87" t="str">
-        <v>Part: CJ1W-EIP21 | Brand: OMRON (Line ADC)</v>
-      </c>
-      <c r="H87">
-        <v>21</v>
-      </c>
-      <c r="I87" t="str">
-        <v>EA</v>
-      </c>
-      <c r="K87">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88" xml:space="preserve">
-      <c r="A88" t="str">
-        <v>TAX-2608-001</v>
-      </c>
-      <c r="B88" t="str">
-        <v>TAX_INVOICE</v>
-      </c>
-      <c r="C88" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="E88">
-        <v>2</v>
-      </c>
-      <c r="F88" t="str">
-        <v/>
-      </c>
-      <c r="G88" t="str" xml:space="preserve">
+      <c r="G87" t="str" xml:space="preserve">
         <v xml:space="preserve">ประกอบด้วย:
 • 2.1 PLC POWER SUPPLY UNIT (CJ1W-PA202 OMRON) 6 EA
 • 2.2 MODULE LINK RACK UNIT (CJ1W-IC101 OMRON) 6 EA
 • 2.3 MODULE LINK RACK UNIT (CJ1W-II101 OMRON) 6 EA
 • 2.4 CABLE LINK RACK (CS1W-CN223 2M OMRON) 6 EA</v>
       </c>
+      <c r="H87">
+        <v>6</v>
+      </c>
+      <c r="I87" t="str">
+        <v>SET</v>
+      </c>
+      <c r="K87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" xml:space="preserve">
+      <c r="A88" t="str">
+        <v>TAX-2608-001</v>
+      </c>
+      <c r="B88" t="str">
+        <v>TAX_INVOICE</v>
+      </c>
+      <c r="C88" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="E88">
+        <v>3</v>
+      </c>
+      <c r="F88" t="str">
+        <v/>
+      </c>
+      <c r="G88" t="str" xml:space="preserve">
+        <v xml:space="preserve">ประกอบด้วย:
+• 3.1 SWITCHING HUB (CBS110-24T-EU CISCO) 1 EA
+• 3.2 ตู้เซิร์ฟเวอร์เครือข่าย 12U (ACR-12U-W APOLLO) 1 EA</v>
+      </c>
       <c r="H88">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I88" t="str">
-        <v>SET</v>
+        <v>EA</v>
       </c>
       <c r="K88">
         <v>0</v>
@@ -5684,43 +5607,12 @@
         <v>2026-08-20</v>
       </c>
       <c r="E89">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F89" t="str">
         <v/>
       </c>
       <c r="G89" t="str" xml:space="preserve">
-        <v xml:space="preserve">ประกอบด้วย:
-• 3.1 SWITCHING HUB (CBS110-24T-EU CISCO) 1 EA
-• 3.2 ตู้เซิร์ฟเวอร์เครือข่าย 12U (ACR-12U-W APOLLO) 1 EA</v>
-      </c>
-      <c r="H89">
-        <v>1</v>
-      </c>
-      <c r="I89" t="str">
-        <v>EA</v>
-      </c>
-      <c r="K89">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="90" xml:space="preserve">
-      <c r="A90" t="str">
-        <v>TAX-2608-001</v>
-      </c>
-      <c r="B90" t="str">
-        <v>TAX_INVOICE</v>
-      </c>
-      <c r="C90" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="E90">
-        <v>4</v>
-      </c>
-      <c r="F90" t="str">
-        <v/>
-      </c>
-      <c r="G90" t="str" xml:space="preserve">
         <v xml:space="preserve">ประกอบด้วย:
 • 4.1 BOX CONTROL (CE-01 TEMCO) 1 EA
 • 4.2 POWER SUPPLY PLC (CJ1W-PA202 OMRON) 1 EA
@@ -5728,6 +5620,36 @@
 • 4.4 INPUT MODULE (CJ1W-211 OMRON) 1 EA
 • 4.5 CIRCUIT PROTECTION (CP30-B 5A FUJI) 1 EA</v>
       </c>
+      <c r="H89">
+        <v>1</v>
+      </c>
+      <c r="I89" t="str">
+        <v>SET</v>
+      </c>
+      <c r="K89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" xml:space="preserve">
+      <c r="A90" t="str">
+        <v>TAX-2608-001</v>
+      </c>
+      <c r="B90" t="str">
+        <v>TAX_INVOICE</v>
+      </c>
+      <c r="C90" t="str">
+        <v>2026-08-20</v>
+      </c>
+      <c r="E90">
+        <v>5</v>
+      </c>
+      <c r="F90" t="str">
+        <v/>
+      </c>
+      <c r="G90" t="str" xml:space="preserve">
+        <v xml:space="preserve">ประกอบด้วย:
+• 5.1 Aluminium profile (LOCAL) 1 SET</v>
+      </c>
       <c r="H90">
         <v>1</v>
       </c>
@@ -5749,52 +5671,51 @@
         <v>2026-08-20</v>
       </c>
       <c r="E91">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F91" t="str">
         <v/>
       </c>
       <c r="G91" t="str" xml:space="preserve">
-        <v xml:space="preserve">ประกอบด้วย:
-• 5.1 Aluminium profile (LOCAL) 1 SET</v>
-      </c>
-      <c r="H91">
-        <v>1</v>
-      </c>
-      <c r="I91" t="str">
-        <v>SET</v>
-      </c>
-      <c r="K91">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="92" xml:space="preserve">
-      <c r="A92" t="str">
-        <v>TAX-2608-001</v>
-      </c>
-      <c r="B92" t="str">
-        <v>TAX_INVOICE</v>
-      </c>
-      <c r="C92" t="str">
-        <v>2026-08-20</v>
-      </c>
-      <c r="E92">
-        <v>6</v>
-      </c>
-      <c r="F92" t="str">
-        <v/>
-      </c>
-      <c r="G92" t="str" xml:space="preserve">
         <v xml:space="preserve">ประกอบด้วย:
 • 6.1 คอมพิวเตอร์ประกอบ (WG-93342286-SO26008123) 1 SET
 • 6.2 เครื่องสำรองไฟ UPS (ZIRCON AX 1000VA/550W) 1 EA
 • 6.3 MOUSE + KEYBOARD (MK120 CORDED LOGITECH) 1 EA</v>
       </c>
+      <c r="H91">
+        <v>1</v>
+      </c>
+      <c r="I91" t="str">
+        <v>SET</v>
+      </c>
+      <c r="K91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>PO-2609-001</v>
+      </c>
+      <c r="B92" t="str">
+        <v>PURCHASE_ORDER</v>
+      </c>
+      <c r="C92" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="E92">
+        <v>1</v>
+      </c>
+      <c r="F92" t="str">
+        <v/>
+      </c>
+      <c r="G92" t="str">
+        <v>Roller Paper Printer Spindle (แกนหมุนกระดาษเครื่องพิมพ์อัปเกรด)</v>
+      </c>
       <c r="H92">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="I92" t="str">
-        <v>SET</v>
+        <v>Set</v>
       </c>
       <c r="K92">
         <v>0</v>
@@ -5811,13 +5732,13 @@
         <v>2026-09-24</v>
       </c>
       <c r="E93">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F93" t="str">
         <v/>
       </c>
       <c r="G93" t="str">
-        <v>Roller Paper Printer Spindle (แกนหมุนกระดาษเครื่องพิมพ์อัปเกรด)</v>
+        <v>mini junction box</v>
       </c>
       <c r="H93">
         <v>15</v>
@@ -5829,38 +5750,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" t="str">
-        <v>PO-2609-001</v>
-      </c>
-      <c r="B94" t="str">
-        <v>PURCHASE_ORDER</v>
-      </c>
-      <c r="C94" t="str">
-        <v>2026-09-24</v>
-      </c>
-      <c r="E94">
-        <v>2</v>
-      </c>
-      <c r="F94" t="str">
-        <v/>
-      </c>
-      <c r="G94" t="str">
-        <v>mini junction box</v>
-      </c>
-      <c r="H94">
-        <v>15</v>
-      </c>
-      <c r="I94" t="str">
-        <v>Set</v>
-      </c>
-      <c r="K94">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L93"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>